<commit_message>
fix norep option in bfm
</commit_message>
<xml_diff>
--- a/output/bfm_summary/bfm_norep_pre/merging_points_wages.xlsx
+++ b/output/bfm_summary/bfm_norep_pre/merging_points_wages.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="196">
   <si>
     <t>p</t>
   </si>
@@ -657,25 +657,25 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>147</v>
+        <v>189</v>
       </c>
       <c r="B1" t="s">
-        <v>148</v>
+        <v>190</v>
       </c>
       <c r="C1" t="s">
-        <v>149</v>
+        <v>191</v>
       </c>
       <c r="D1" t="s">
-        <v>150</v>
+        <v>192</v>
       </c>
       <c r="E1" t="s">
-        <v>151</v>
+        <v>193</v>
       </c>
       <c r="F1" t="s">
-        <v>152</v>
+        <v>194</v>
       </c>
       <c r="G1" t="s">
-        <v>153</v>
+        <v>195</v>
       </c>
     </row>
     <row r="2">
@@ -1652,50 +1652,50 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G51"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>154</v>
+        <v>189</v>
       </c>
       <c r="B1" t="s">
-        <v>155</v>
+        <v>190</v>
       </c>
       <c r="C1" t="s">
-        <v>156</v>
+        <v>191</v>
       </c>
       <c r="D1" t="s">
-        <v>157</v>
+        <v>192</v>
       </c>
       <c r="E1" t="s">
-        <v>158</v>
+        <v>193</v>
       </c>
       <c r="F1" t="s">
-        <v>159</v>
+        <v>194</v>
       </c>
       <c r="G1" t="s">
-        <v>160</v>
+        <v>195</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1">
-        <v>0.76999998092651367</v>
+        <v>0.75999999046325684</v>
       </c>
       <c r="B2" s="1">
-        <v>0.98037236928939819</v>
+        <v>0.98703926801681519</v>
       </c>
       <c r="C2" s="1">
-        <v>0.6906282901763916</v>
+        <v>0.47368142008781433</v>
       </c>
       <c r="D2" s="1">
-        <v>1.2400661706924438</v>
+        <v>1.1305828094482422</v>
       </c>
       <c r="E2" s="1">
         <v>0</v>
       </c>
       <c r="F2" s="1">
-        <v>204000</v>
+        <v>0.11999999731779099</v>
       </c>
       <c r="G2" s="1">
         <v>0.98000001907348633</v>
@@ -1703,139 +1703,139 @@
     </row>
     <row r="3">
       <c r="A3" s="1">
-        <v>0.77999997138977051</v>
+        <v>0.76999998092651367</v>
       </c>
       <c r="B3" s="1">
-        <v>0.9766576886177063</v>
+        <v>0.98037236928939819</v>
       </c>
       <c r="C3" s="1">
-        <v>0.73808306455612183</v>
+        <v>0.6906282901763916</v>
       </c>
       <c r="D3" s="1">
-        <v>1.2400661706924438</v>
+        <v>1.1305828094482422</v>
       </c>
       <c r="E3" s="1">
         <v>0</v>
       </c>
       <c r="F3" s="1">
-        <v>1184400</v>
+        <v>204000</v>
       </c>
       <c r="G3" s="1"/>
     </row>
     <row r="4">
       <c r="A4" s="1">
-        <v>0.79000002145767212</v>
+        <v>0.77999997138977051</v>
       </c>
       <c r="B4" s="1">
-        <v>0.97363770008087158</v>
+        <v>0.9766576886177063</v>
       </c>
       <c r="C4" s="1">
-        <v>1.3372215032577515</v>
+        <v>0.73808306455612183</v>
       </c>
       <c r="D4" s="1">
-        <v>1.2400661706924438</v>
+        <v>1.1305828094482422</v>
       </c>
       <c r="E4" s="1">
         <v>0</v>
       </c>
       <c r="F4" s="1">
-        <v>1560000</v>
+        <v>1184400</v>
       </c>
       <c r="G4" s="1"/>
     </row>
     <row r="5">
       <c r="A5" s="1">
-        <v>0.80000001192092896</v>
+        <v>0.79000002145767212</v>
       </c>
       <c r="B5" s="1">
-        <v>0.97818249464035034</v>
+        <v>0.97363770008087158</v>
       </c>
       <c r="C5" s="1">
-        <v>1.4630857706069946</v>
+        <v>1.3372215032577515</v>
       </c>
       <c r="D5" s="1">
-        <v>1.2400661706924438</v>
+        <v>1.1305828094482422</v>
       </c>
       <c r="E5" s="1">
         <v>0</v>
       </c>
       <c r="F5" s="1">
-        <v>2040000</v>
+        <v>1560000</v>
       </c>
       <c r="G5" s="1"/>
     </row>
     <row r="6">
       <c r="A6" s="1">
-        <v>0.81000000238418579</v>
+        <v>0.80000001192092896</v>
       </c>
       <c r="B6" s="1">
-        <v>0.98416894674301147</v>
+        <v>0.97818249464035034</v>
       </c>
       <c r="C6" s="1">
-        <v>1.7332562208175659</v>
+        <v>1.4630857706069946</v>
       </c>
       <c r="D6" s="1">
-        <v>1.2400661706924438</v>
+        <v>1.1305828094482422</v>
       </c>
       <c r="E6" s="1">
         <v>0</v>
       </c>
       <c r="F6" s="1">
-        <v>2366788.5</v>
+        <v>2040000</v>
       </c>
       <c r="G6" s="1"/>
     </row>
     <row r="7">
       <c r="A7" s="1">
-        <v>0.81999999284744263</v>
+        <v>0.81000000238418579</v>
       </c>
       <c r="B7" s="1">
-        <v>0.99330413341522217</v>
+        <v>0.98416894674301147</v>
       </c>
       <c r="C7" s="1">
-        <v>1.4781253337860107</v>
+        <v>1.7332562208175659</v>
       </c>
       <c r="D7" s="1">
-        <v>1.2400661706924438</v>
+        <v>1.1305828094482422</v>
       </c>
       <c r="E7" s="1">
         <v>0</v>
       </c>
       <c r="F7" s="1">
-        <v>2609070.25</v>
+        <v>2366788.5</v>
       </c>
       <c r="G7" s="1"/>
     </row>
     <row r="8">
       <c r="A8" s="1">
-        <v>0.82999998331069946</v>
+        <v>0.81999999284744263</v>
       </c>
       <c r="B8" s="1">
-        <v>0.99914532899856567</v>
+        <v>0.99330413341522217</v>
       </c>
       <c r="C8" s="1">
-        <v>0.90785688161849976</v>
+        <v>1.4781253337860107</v>
       </c>
       <c r="D8" s="1">
-        <v>1.0490860939025879</v>
+        <v>1.1305828094482422</v>
       </c>
       <c r="E8" s="1">
         <v>0</v>
       </c>
       <c r="F8" s="1">
-        <v>2758320</v>
+        <v>2609070.25</v>
       </c>
       <c r="G8" s="1"/>
     </row>
     <row r="9">
       <c r="A9" s="1">
-        <v>0.8399999737739563</v>
+        <v>0.82999998331069946</v>
       </c>
       <c r="B9" s="1">
-        <v>0.99805861711502075</v>
+        <v>0.99914532899856567</v>
       </c>
       <c r="C9" s="1">
-        <v>0.73520088195800781</v>
+        <v>0.90785688161849976</v>
       </c>
       <c r="D9" s="1">
         <v>1.0490860939025879</v>
@@ -1844,19 +1844,19 @@
         <v>0</v>
       </c>
       <c r="F9" s="1">
-        <v>2893920</v>
+        <v>2758320</v>
       </c>
       <c r="G9" s="1"/>
     </row>
     <row r="10">
       <c r="A10" s="1">
-        <v>0.85000002384185791</v>
+        <v>0.8399999737739563</v>
       </c>
       <c r="B10" s="1">
-        <v>0.99496614933013916</v>
+        <v>0.99805861711502075</v>
       </c>
       <c r="C10" s="1">
-        <v>0.99141967296600342</v>
+        <v>0.73520088195800781</v>
       </c>
       <c r="D10" s="1">
         <v>1.0490860939025879</v>
@@ -1865,19 +1865,19 @@
         <v>0</v>
       </c>
       <c r="F10" s="1">
-        <v>3000000</v>
+        <v>2893920</v>
       </c>
       <c r="G10" s="1"/>
     </row>
     <row r="11">
       <c r="A11" s="1">
-        <v>0.86000001430511475</v>
+        <v>0.85000002384185791</v>
       </c>
       <c r="B11" s="1">
-        <v>0.99492484331130981</v>
+        <v>0.99496614933013916</v>
       </c>
       <c r="C11" s="1">
-        <v>1.1073371171951294</v>
+        <v>0.99141967296600342</v>
       </c>
       <c r="D11" s="1">
         <v>1.0490860939025879</v>
@@ -1886,19 +1886,19 @@
         <v>0</v>
       </c>
       <c r="F11" s="1">
-        <v>3187719.75</v>
+        <v>3000000</v>
       </c>
       <c r="G11" s="1"/>
     </row>
     <row r="12">
       <c r="A12" s="1">
-        <v>0.87000000476837158</v>
+        <v>0.86000001430511475</v>
       </c>
       <c r="B12" s="1">
-        <v>0.99621701240539551</v>
+        <v>0.99492484331130981</v>
       </c>
       <c r="C12" s="1">
-        <v>1.2705185413360596</v>
+        <v>1.1073371171951294</v>
       </c>
       <c r="D12" s="1">
         <v>1.0490860939025879</v>
@@ -1907,19 +1907,19 @@
         <v>0</v>
       </c>
       <c r="F12" s="1">
-        <v>3397248</v>
+        <v>3187719.75</v>
       </c>
       <c r="G12" s="1"/>
     </row>
     <row r="13">
       <c r="A13" s="1">
-        <v>0.87999999523162842</v>
+        <v>0.87000000476837158</v>
       </c>
       <c r="B13" s="1">
-        <v>0.99933403730392456</v>
+        <v>0.99621701240539551</v>
       </c>
       <c r="C13" s="1">
-        <v>1.1511121988296509</v>
+        <v>1.2705185413360596</v>
       </c>
       <c r="D13" s="1">
         <v>1.0490860939025879</v>
@@ -1928,19 +1928,19 @@
         <v>0</v>
       </c>
       <c r="F13" s="1">
-        <v>3616610.25</v>
+        <v>3397248</v>
       </c>
       <c r="G13" s="1"/>
     </row>
     <row r="14">
       <c r="A14" s="1">
-        <v>0.88999998569488525</v>
+        <v>0.87999999523162842</v>
       </c>
       <c r="B14" s="1">
-        <v>1.0010395050048828</v>
+        <v>0.99933403730392456</v>
       </c>
       <c r="C14" s="1">
-        <v>1.0480890274047852</v>
+        <v>1.1511121988296509</v>
       </c>
       <c r="D14" s="1">
         <v>1.0490860939025879</v>
@@ -1949,19 +1949,19 @@
         <v>0</v>
       </c>
       <c r="F14" s="1">
-        <v>3902580</v>
+        <v>3616610.25</v>
       </c>
       <c r="G14" s="1"/>
     </row>
     <row r="15">
       <c r="A15" s="1">
-        <v>0.89999997615814209</v>
+        <v>0.88999998569488525</v>
       </c>
       <c r="B15" s="1">
-        <v>1.0015621185302734</v>
+        <v>1.0010395050048828</v>
       </c>
       <c r="C15" s="1">
-        <v>0.98395907878875732</v>
+        <v>1.0480890274047852</v>
       </c>
       <c r="D15" s="1">
         <v>1.0490860939025879</v>
@@ -1970,19 +1970,19 @@
         <v>0</v>
       </c>
       <c r="F15" s="1">
-        <v>4236000</v>
+        <v>3902580</v>
       </c>
       <c r="G15" s="1"/>
     </row>
     <row r="16">
       <c r="A16" s="1">
-        <v>0.9100000262260437</v>
+        <v>0.89999997615814209</v>
       </c>
       <c r="B16" s="1">
-        <v>1.0013687610626221</v>
+        <v>1.0015621185302734</v>
       </c>
       <c r="C16" s="1">
-        <v>1.1098942756652832</v>
+        <v>0.98395907878875732</v>
       </c>
       <c r="D16" s="1">
         <v>1.0490860939025879</v>
@@ -1991,19 +1991,19 @@
         <v>0</v>
       </c>
       <c r="F16" s="1">
-        <v>4635300</v>
+        <v>4236000</v>
       </c>
       <c r="G16" s="1"/>
     </row>
     <row r="17">
       <c r="A17" s="1">
-        <v>0.92000001668930054</v>
+        <v>0.9100000262260437</v>
       </c>
       <c r="B17" s="1">
-        <v>1.0025483369827271</v>
+        <v>1.0013687610626221</v>
       </c>
       <c r="C17" s="1">
-        <v>0.99497371912002563</v>
+        <v>1.1098942756652832</v>
       </c>
       <c r="D17" s="1">
         <v>1.0490860939025879</v>
@@ -2012,19 +2012,19 @@
         <v>0</v>
       </c>
       <c r="F17" s="1">
-        <v>5085276</v>
+        <v>4635300</v>
       </c>
       <c r="G17" s="1"/>
     </row>
     <row r="18">
       <c r="A18" s="1">
-        <v>0.93000000715255737</v>
+        <v>0.92000001668930054</v>
       </c>
       <c r="B18" s="1">
-        <v>1.0024669170379639</v>
+        <v>1.0025483369827271</v>
       </c>
       <c r="C18" s="1">
-        <v>1.122333288192749</v>
+        <v>0.99497371912002563</v>
       </c>
       <c r="D18" s="1">
         <v>1.0490860939025879</v>
@@ -2033,19 +2033,19 @@
         <v>0</v>
       </c>
       <c r="F18" s="1">
-        <v>5646960</v>
+        <v>5085276</v>
       </c>
       <c r="G18" s="1"/>
     </row>
     <row r="19">
       <c r="A19" s="1">
-        <v>0.93999999761581421</v>
+        <v>0.93000000715255737</v>
       </c>
       <c r="B19" s="1">
-        <v>1.0037420988082886</v>
+        <v>1.0024669170379639</v>
       </c>
       <c r="C19" s="1">
-        <v>1.114748477935791</v>
+        <v>1.122333288192749</v>
       </c>
       <c r="D19" s="1">
         <v>1.0490860939025879</v>
@@ -2054,19 +2054,19 @@
         <v>0</v>
       </c>
       <c r="F19" s="1">
-        <v>6360624</v>
+        <v>5646960</v>
       </c>
       <c r="G19" s="1"/>
     </row>
     <row r="20">
       <c r="A20" s="1">
-        <v>0.94999998807907104</v>
+        <v>0.93999999761581421</v>
       </c>
       <c r="B20" s="1">
-        <v>1.0049105882644653</v>
+        <v>1.0037420988082886</v>
       </c>
       <c r="C20" s="1">
-        <v>0.99902617931365967</v>
+        <v>1.114748477935791</v>
       </c>
       <c r="D20" s="1">
         <v>1.0490860939025879</v>
@@ -2075,19 +2075,19 @@
         <v>0</v>
       </c>
       <c r="F20" s="1">
-        <v>7356000</v>
+        <v>6360624</v>
       </c>
       <c r="G20" s="1"/>
     </row>
     <row r="21">
       <c r="A21" s="1">
-        <v>0.95999997854232788</v>
+        <v>0.94999998807907104</v>
       </c>
       <c r="B21" s="1">
-        <v>1.0048493146896362</v>
+        <v>1.0049105882644653</v>
       </c>
       <c r="C21" s="1">
-        <v>1.150736927986145</v>
+        <v>0.99902617931365967</v>
       </c>
       <c r="D21" s="1">
         <v>1.0490860939025879</v>
@@ -2096,61 +2096,61 @@
         <v>0</v>
       </c>
       <c r="F21" s="1">
-        <v>8659777</v>
+        <v>7356000</v>
       </c>
       <c r="G21" s="1"/>
     </row>
     <row r="22">
       <c r="A22" s="1">
-        <v>0.97000002861022949</v>
+        <v>0.95999997854232788</v>
       </c>
       <c r="B22" s="1">
-        <v>1.0063532590866089</v>
+        <v>1.0048493146896362</v>
       </c>
       <c r="C22" s="1">
-        <v>1.0155394077301025</v>
+        <v>1.150736927986145</v>
       </c>
       <c r="D22" s="1">
-        <v>1.0155394077301025</v>
+        <v>1.0490860939025879</v>
       </c>
       <c r="E22" s="1">
         <v>0</v>
       </c>
       <c r="F22" s="1">
-        <v>10445760</v>
+        <v>8659777</v>
       </c>
       <c r="G22" s="1"/>
     </row>
     <row r="23">
       <c r="A23" s="1">
-        <v>0.98000001907348633</v>
+        <v>0.97000002861022949</v>
       </c>
       <c r="B23" s="1">
-        <v>1.0064470767974854</v>
+        <v>1.0063532590866089</v>
       </c>
       <c r="C23" s="1">
-        <v>0.75239020586013794</v>
+        <v>1.0155394077301025</v>
       </c>
       <c r="D23" s="1">
-        <v>0.78848767280578613</v>
+        <v>1.0155394077301025</v>
       </c>
       <c r="E23" s="1">
         <v>0</v>
       </c>
       <c r="F23" s="1">
-        <v>13056165</v>
+        <v>10445760</v>
       </c>
       <c r="G23" s="1"/>
     </row>
     <row r="24">
       <c r="A24" s="1">
-        <v>0.99000000953674316</v>
+        <v>0.98000001907348633</v>
       </c>
       <c r="B24" s="1">
-        <v>1.0038808584213257</v>
+        <v>1.0064470767974854</v>
       </c>
       <c r="C24" s="1">
-        <v>1.0196256637573242</v>
+        <v>0.75239020586013794</v>
       </c>
       <c r="D24" s="1">
         <v>0.78848767280578613</v>
@@ -2159,19 +2159,19 @@
         <v>0</v>
       </c>
       <c r="F24" s="1">
-        <v>18095660</v>
+        <v>13056165</v>
       </c>
       <c r="G24" s="1"/>
     </row>
     <row r="25">
       <c r="A25" s="1">
-        <v>0.99099999666213989</v>
+        <v>0.99000000953674316</v>
       </c>
       <c r="B25" s="1">
-        <v>1.0038967132568359</v>
+        <v>1.0038808584213257</v>
       </c>
       <c r="C25" s="1">
-        <v>0.68935799598693848</v>
+        <v>1.0196256637573242</v>
       </c>
       <c r="D25" s="1">
         <v>0.78848767280578613</v>
@@ -2180,19 +2180,19 @@
         <v>0</v>
       </c>
       <c r="F25" s="1">
-        <v>18996832</v>
+        <v>18095660</v>
       </c>
       <c r="G25" s="1"/>
     </row>
     <row r="26">
       <c r="A26" s="1">
-        <v>0.99199998378753662</v>
+        <v>0.99099999666213989</v>
       </c>
       <c r="B26" s="1">
-        <v>1.0035796165466309</v>
+        <v>1.0038967132568359</v>
       </c>
       <c r="C26" s="1">
-        <v>1.0174585580825806</v>
+        <v>0.68935799598693848</v>
       </c>
       <c r="D26" s="1">
         <v>0.78848767280578613</v>
@@ -2201,40 +2201,40 @@
         <v>0</v>
       </c>
       <c r="F26" s="1">
-        <v>19997736</v>
+        <v>18996832</v>
       </c>
       <c r="G26" s="1"/>
     </row>
     <row r="27">
       <c r="A27" s="1">
-        <v>0.99299997091293335</v>
+        <v>0.99199998378753662</v>
       </c>
       <c r="B27" s="1">
-        <v>1.0035936832427979</v>
+        <v>1.0035796165466309</v>
       </c>
       <c r="C27" s="1">
-        <v>0.60177075862884521</v>
+        <v>1.0174585580825806</v>
       </c>
       <c r="D27" s="1">
-        <v>0.73275786638259888</v>
+        <v>0.78848767280578613</v>
       </c>
       <c r="E27" s="1">
         <v>0</v>
       </c>
       <c r="F27" s="1">
-        <v>21186084</v>
+        <v>19997736</v>
       </c>
       <c r="G27" s="1"/>
     </row>
     <row r="28">
       <c r="A28" s="1">
-        <v>0.99400001764297485</v>
+        <v>0.99299997091293335</v>
       </c>
       <c r="B28" s="1">
-        <v>1.0031893253326416</v>
+        <v>1.0035936832427979</v>
       </c>
       <c r="C28" s="1">
-        <v>0.76694053411483765</v>
+        <v>0.60177075862884521</v>
       </c>
       <c r="D28" s="1">
         <v>0.73275786638259888</v>
@@ -2243,19 +2243,19 @@
         <v>0</v>
       </c>
       <c r="F28" s="1">
-        <v>22707424</v>
+        <v>21186084</v>
       </c>
       <c r="G28" s="1"/>
     </row>
     <row r="29">
       <c r="A29" s="1">
-        <v>0.99500000476837158</v>
+        <v>0.99400001764297485</v>
       </c>
       <c r="B29" s="1">
-        <v>1.0029518604278564</v>
+        <v>1.0031893253326416</v>
       </c>
       <c r="C29" s="1">
-        <v>0.82957005500793457</v>
+        <v>0.76694053411483765</v>
       </c>
       <c r="D29" s="1">
         <v>0.73275786638259888</v>
@@ -2264,61 +2264,61 @@
         <v>0</v>
       </c>
       <c r="F29" s="1">
-        <v>24684000</v>
+        <v>22707424</v>
       </c>
       <c r="G29" s="1"/>
     </row>
     <row r="30">
       <c r="A30" s="1">
-        <v>0.99599999189376831</v>
+        <v>0.99500000476837158</v>
       </c>
       <c r="B30" s="1">
-        <v>1.0027778148651123</v>
+        <v>1.0029518604278564</v>
       </c>
       <c r="C30" s="1">
-        <v>0.37621045112609863</v>
+        <v>0.82957005500793457</v>
       </c>
       <c r="D30" s="1">
-        <v>0.37621045112609863</v>
+        <v>0.73275786638259888</v>
       </c>
       <c r="E30" s="1">
         <v>0</v>
       </c>
       <c r="F30" s="1">
-        <v>27138690</v>
+        <v>24684000</v>
       </c>
       <c r="G30" s="1"/>
     </row>
     <row r="31">
       <c r="A31" s="1">
-        <v>0.99699997901916504</v>
+        <v>0.99599999189376831</v>
       </c>
       <c r="B31" s="1">
-        <v>1.0021494626998901</v>
+        <v>1.0027778148651123</v>
       </c>
       <c r="C31" s="1">
-        <v>0.30099374055862427</v>
+        <v>0.37621045112609863</v>
       </c>
       <c r="D31" s="1">
-        <v>0.31214693188667297</v>
+        <v>0.37621045112609863</v>
       </c>
       <c r="E31" s="1">
         <v>0</v>
       </c>
       <c r="F31" s="1">
-        <v>30177476</v>
+        <v>27138690</v>
       </c>
       <c r="G31" s="1"/>
     </row>
     <row r="32">
       <c r="A32" s="1">
-        <v>0.99800002574920654</v>
+        <v>0.99699997901916504</v>
       </c>
       <c r="B32" s="1">
-        <v>1.0014468431472778</v>
+        <v>1.0021494626998901</v>
       </c>
       <c r="C32" s="1">
-        <v>0.29147642850875854</v>
+        <v>0.30099374055862427</v>
       </c>
       <c r="D32" s="1">
         <v>0.31214693188667297</v>
@@ -2327,19 +2327,19 @@
         <v>0</v>
       </c>
       <c r="F32" s="1">
-        <v>34623384</v>
+        <v>30177476</v>
       </c>
       <c r="G32" s="1"/>
     </row>
     <row r="33">
       <c r="A33" s="1">
-        <v>0.99900001287460327</v>
+        <v>0.99800002574920654</v>
       </c>
       <c r="B33" s="1">
-        <v>1.0007361173629761</v>
+        <v>1.0014468431472778</v>
       </c>
       <c r="C33" s="1">
-        <v>0.18200476467609406</v>
+        <v>0.29147642850875854</v>
       </c>
       <c r="D33" s="1">
         <v>0.31214693188667297</v>
@@ -2348,19 +2348,19 @@
         <v>0</v>
       </c>
       <c r="F33" s="1">
-        <v>44293144</v>
+        <v>34623384</v>
       </c>
       <c r="G33" s="1"/>
     </row>
     <row r="34">
       <c r="A34" s="1">
-        <v>0.99910002946853638</v>
+        <v>0.99900001287460327</v>
       </c>
       <c r="B34" s="1">
-        <v>1.0009007453918457</v>
+        <v>1.0007361173629761</v>
       </c>
       <c r="C34" s="1">
-        <v>0</v>
+        <v>0.18200476467609406</v>
       </c>
       <c r="D34" s="1">
         <v>0.31214693188667297</v>
@@ -2369,19 +2369,19 @@
         <v>0</v>
       </c>
       <c r="F34" s="1">
-        <v>46035348</v>
+        <v>44293144</v>
       </c>
       <c r="G34" s="1"/>
     </row>
     <row r="35">
       <c r="A35" s="1">
-        <v>0.99919998645782471</v>
+        <v>0.99910002946853638</v>
       </c>
       <c r="B35" s="1">
-        <v>1.000554084777832</v>
+        <v>1.0009007453918457</v>
       </c>
       <c r="C35" s="1">
-        <v>0.34450903534889221</v>
+        <v>0</v>
       </c>
       <c r="D35" s="1">
         <v>0.31214693188667297</v>
@@ -2390,19 +2390,19 @@
         <v>0</v>
       </c>
       <c r="F35" s="1">
-        <v>48166996</v>
+        <v>46035348</v>
       </c>
       <c r="G35" s="1"/>
     </row>
     <row r="36">
       <c r="A36" s="1">
-        <v>0.99930000305175781</v>
+        <v>0.99919998645782471</v>
       </c>
       <c r="B36" s="1">
-        <v>1.0004884004592896</v>
+        <v>1.000554084777832</v>
       </c>
       <c r="C36" s="1">
-        <v>0.071501873433589935</v>
+        <v>0.34450903534889221</v>
       </c>
       <c r="D36" s="1">
         <v>0.31214693188667297</v>
@@ -2411,19 +2411,19 @@
         <v>0</v>
       </c>
       <c r="F36" s="1">
-        <v>50713824</v>
+        <v>48166996</v>
       </c>
       <c r="G36" s="1"/>
     </row>
     <row r="37">
       <c r="A37" s="1">
-        <v>0.99940001964569092</v>
+        <v>0.99930000305175781</v>
       </c>
       <c r="B37" s="1">
-        <v>1.0003954172134399</v>
+        <v>1.0004884004592896</v>
       </c>
       <c r="C37" s="1">
-        <v>1.2812972068786621</v>
+        <v>0.071501873433589935</v>
       </c>
       <c r="D37" s="1">
         <v>0.31214693188667297</v>
@@ -2432,40 +2432,40 @@
         <v>0</v>
       </c>
       <c r="F37" s="1">
-        <v>53721440</v>
+        <v>50713824</v>
       </c>
       <c r="G37" s="1"/>
     </row>
     <row r="38">
       <c r="A38" s="1">
-        <v>0.99949997663497925</v>
+        <v>0.99940001964569092</v>
       </c>
       <c r="B38" s="1">
-        <v>1.0005003213882446</v>
+        <v>1.0003954172134399</v>
       </c>
       <c r="C38" s="1">
-        <v>0</v>
+        <v>1.2812972068786621</v>
       </c>
       <c r="D38" s="1">
-        <v>0.29034093022346497</v>
+        <v>0.31214693188667297</v>
       </c>
       <c r="E38" s="1">
         <v>0</v>
       </c>
       <c r="F38" s="1">
-        <v>57226288</v>
+        <v>53721440</v>
       </c>
       <c r="G38" s="1"/>
     </row>
     <row r="39">
       <c r="A39" s="1">
-        <v>0.99959999322891235</v>
+        <v>0.99949997663497925</v>
       </c>
       <c r="B39" s="1">
-        <v>1.0003234148025513</v>
+        <v>1.0005003213882446</v>
       </c>
       <c r="C39" s="1">
-        <v>0.58068186044692993</v>
+        <v>0</v>
       </c>
       <c r="D39" s="1">
         <v>0.29034093022346497</v>
@@ -2474,58 +2474,58 @@
         <v>0</v>
       </c>
       <c r="F39" s="1">
-        <v>61417188</v>
+        <v>57226288</v>
       </c>
       <c r="G39" s="1"/>
     </row>
     <row r="40">
       <c r="A40" s="1">
-        <v>0.99970000982284546</v>
+        <v>0.99959999322891235</v>
       </c>
       <c r="B40" s="1">
-        <v>1.0002814531326294</v>
+        <v>1.0003234148025513</v>
       </c>
       <c r="C40" s="1">
-        <v>0.18633821606636047</v>
+        <v>0.58068186044692993</v>
       </c>
       <c r="D40" s="1">
-        <v>0.18633821606636047</v>
+        <v>0.29034093022346497</v>
       </c>
       <c r="E40" s="1">
         <v>0</v>
       </c>
       <c r="F40" s="1">
-        <v>67407672</v>
+        <v>61417188</v>
       </c>
       <c r="G40" s="1"/>
     </row>
     <row r="41">
       <c r="A41" s="1">
-        <v>0.99980002641677856</v>
+        <v>0.99970000982284546</v>
       </c>
       <c r="B41" s="1">
-        <v>1.0002000331878662</v>
+        <v>1.0002814531326294</v>
       </c>
       <c r="C41" s="1">
-        <v>0</v>
+        <v>0.18633821606636047</v>
       </c>
       <c r="D41" s="1">
-        <v>0</v>
+        <v>0.18633821606636047</v>
       </c>
       <c r="E41" s="1">
         <v>0</v>
       </c>
       <c r="F41" s="1">
-        <v>76822680</v>
+        <v>67407672</v>
       </c>
       <c r="G41" s="1"/>
     </row>
     <row r="42">
       <c r="A42" s="1">
-        <v>0.99989998340606689</v>
+        <v>0.99980002641677856</v>
       </c>
       <c r="B42" s="1">
-        <v>1.0001000165939331</v>
+        <v>1.0002000331878662</v>
       </c>
       <c r="C42" s="1">
         <v>0</v>
@@ -2537,16 +2537,16 @@
         <v>0</v>
       </c>
       <c r="F42" s="1">
-        <v>93302120</v>
+        <v>76822680</v>
       </c>
       <c r="G42" s="1"/>
     </row>
     <row r="43">
       <c r="A43" s="1">
-        <v>0.99990999698638916</v>
+        <v>0.99989998340606689</v>
       </c>
       <c r="B43" s="1">
-        <v>1.0000900030136108</v>
+        <v>1.0001000165939331</v>
       </c>
       <c r="C43" s="1">
         <v>0</v>
@@ -2558,16 +2558,16 @@
         <v>0</v>
       </c>
       <c r="F43" s="1">
-        <v>96582464</v>
+        <v>93302120</v>
       </c>
       <c r="G43" s="1"/>
     </row>
     <row r="44">
       <c r="A44" s="1">
-        <v>0.99992001056671143</v>
+        <v>0.99990999698638916</v>
       </c>
       <c r="B44" s="1">
-        <v>1.0000799894332886</v>
+        <v>1.0000900030136108</v>
       </c>
       <c r="C44" s="1">
         <v>0</v>
@@ -2579,16 +2579,16 @@
         <v>0</v>
       </c>
       <c r="F44" s="1">
-        <v>99827432</v>
+        <v>96582464</v>
       </c>
       <c r="G44" s="1"/>
     </row>
     <row r="45">
       <c r="A45" s="1">
-        <v>0.99993002414703369</v>
+        <v>0.99992001056671143</v>
       </c>
       <c r="B45" s="1">
-        <v>1.0000699758529663</v>
+        <v>1.0000799894332886</v>
       </c>
       <c r="C45" s="1">
         <v>0</v>
@@ -2600,16 +2600,16 @@
         <v>0</v>
       </c>
       <c r="F45" s="1">
-        <v>102645952</v>
+        <v>99827432</v>
       </c>
       <c r="G45" s="1"/>
     </row>
     <row r="46">
       <c r="A46" s="1">
-        <v>0.99993997812271118</v>
+        <v>0.99993002414703369</v>
       </c>
       <c r="B46" s="1">
-        <v>1.0000600814819336</v>
+        <v>1.0000699758529663</v>
       </c>
       <c r="C46" s="1">
         <v>0</v>
@@ -2621,16 +2621,16 @@
         <v>0</v>
       </c>
       <c r="F46" s="1">
-        <v>108249792</v>
+        <v>102645952</v>
       </c>
       <c r="G46" s="1"/>
     </row>
     <row r="47">
       <c r="A47" s="1">
-        <v>0.99994999170303345</v>
+        <v>0.99993997812271118</v>
       </c>
       <c r="B47" s="1">
-        <v>1.0000500679016113</v>
+        <v>1.0000600814819336</v>
       </c>
       <c r="C47" s="1">
         <v>0</v>
@@ -2642,16 +2642,16 @@
         <v>0</v>
       </c>
       <c r="F47" s="1">
-        <v>115354200</v>
+        <v>108249792</v>
       </c>
       <c r="G47" s="1"/>
     </row>
     <row r="48">
       <c r="A48" s="1">
-        <v>0.99996000528335571</v>
+        <v>0.99994999170303345</v>
       </c>
       <c r="B48" s="1">
-        <v>1.0000400543212891</v>
+        <v>1.0000500679016113</v>
       </c>
       <c r="C48" s="1">
         <v>0</v>
@@ -2663,16 +2663,16 @@
         <v>0</v>
       </c>
       <c r="F48" s="1">
-        <v>125994240</v>
+        <v>115354200</v>
       </c>
       <c r="G48" s="1"/>
     </row>
     <row r="49">
       <c r="A49" s="1">
-        <v>0.99997001886367798</v>
+        <v>0.99996000528335571</v>
       </c>
       <c r="B49" s="1">
-        <v>1.0000300407409668</v>
+        <v>1.0000400543212891</v>
       </c>
       <c r="C49" s="1">
         <v>0</v>
@@ -2684,16 +2684,16 @@
         <v>0</v>
       </c>
       <c r="F49" s="1">
-        <v>139355792</v>
+        <v>125994240</v>
       </c>
       <c r="G49" s="1"/>
     </row>
     <row r="50">
       <c r="A50" s="1">
-        <v>0.99997997283935547</v>
+        <v>0.99997001886367798</v>
       </c>
       <c r="B50" s="1">
-        <v>1.0000200271606445</v>
+        <v>1.0000300407409668</v>
       </c>
       <c r="C50" s="1">
         <v>0</v>
@@ -2705,30 +2705,51 @@
         <v>0</v>
       </c>
       <c r="F50" s="1">
-        <v>153453312</v>
+        <v>139355792</v>
       </c>
       <c r="G50" s="1"/>
     </row>
     <row r="51">
       <c r="A51" s="1">
+        <v>0.99997997283935547</v>
+      </c>
+      <c r="B51" s="1">
+        <v>1.0000200271606445</v>
+      </c>
+      <c r="C51" s="1">
+        <v>0</v>
+      </c>
+      <c r="D51" s="1">
+        <v>0</v>
+      </c>
+      <c r="E51" s="1">
+        <v>0</v>
+      </c>
+      <c r="F51" s="1">
+        <v>153453312</v>
+      </c>
+      <c r="G51" s="1"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="1">
         <v>0.99998998641967773</v>
       </c>
-      <c r="B51" s="1">
+      <c r="B52" s="1">
         <v>1.0000100135803223</v>
       </c>
-      <c r="C51" s="1">
-        <v>0</v>
-      </c>
-      <c r="D51" s="1">
-        <v>0</v>
-      </c>
-      <c r="E51" s="1">
-        <v>0</v>
-      </c>
-      <c r="F51" s="1">
+      <c r="C52" s="1">
+        <v>0</v>
+      </c>
+      <c r="D52" s="1">
+        <v>0</v>
+      </c>
+      <c r="E52" s="1">
+        <v>0</v>
+      </c>
+      <c r="F52" s="1">
         <v>191015408</v>
       </c>
-      <c r="G51" s="1"/>
+      <c r="G52" s="1"/>
     </row>
   </sheetData>
 </worksheet>
@@ -2736,50 +2757,50 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G51"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>161</v>
+        <v>189</v>
       </c>
       <c r="B1" t="s">
-        <v>162</v>
+        <v>190</v>
       </c>
       <c r="C1" t="s">
-        <v>163</v>
+        <v>191</v>
       </c>
       <c r="D1" t="s">
-        <v>164</v>
+        <v>192</v>
       </c>
       <c r="E1" t="s">
-        <v>165</v>
+        <v>193</v>
       </c>
       <c r="F1" t="s">
-        <v>166</v>
+        <v>194</v>
       </c>
       <c r="G1" t="s">
-        <v>167</v>
+        <v>195</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1">
-        <v>0.76999998092651367</v>
+        <v>0.75999999046325684</v>
       </c>
       <c r="B2" s="1">
-        <v>0.97337204217910767</v>
+        <v>0.97803968191146851</v>
       </c>
       <c r="C2" s="1">
-        <v>0.74314266443252563</v>
+        <v>0.61863207817077637</v>
       </c>
       <c r="D2" s="1">
-        <v>1.2959392070770264</v>
+        <v>1.1604779958724976</v>
       </c>
       <c r="E2" s="1">
         <v>0</v>
       </c>
       <c r="F2" s="1">
-        <v>814682.0625</v>
+        <v>0.11999999731779099</v>
       </c>
       <c r="G2" s="1">
         <v>0.97000002861022949</v>
@@ -2787,97 +2808,97 @@
     </row>
     <row r="3">
       <c r="A3" s="1">
-        <v>0.77999997138977051</v>
+        <v>0.76999998092651367</v>
       </c>
       <c r="B3" s="1">
-        <v>0.97042042016983032</v>
+        <v>0.97337204217910767</v>
       </c>
       <c r="C3" s="1">
-        <v>0.86818379163742065</v>
+        <v>0.74314266443252563</v>
       </c>
       <c r="D3" s="1">
-        <v>1.2959392070770264</v>
+        <v>1.1604779958724976</v>
       </c>
       <c r="E3" s="1">
         <v>0</v>
       </c>
       <c r="F3" s="1">
-        <v>1446966</v>
+        <v>814682.0625</v>
       </c>
       <c r="G3" s="1"/>
     </row>
     <row r="4">
       <c r="A4" s="1">
-        <v>0.79000002145767212</v>
+        <v>0.77999997138977051</v>
       </c>
       <c r="B4" s="1">
-        <v>0.96912628412246704</v>
+        <v>0.97042042016983032</v>
       </c>
       <c r="C4" s="1">
-        <v>1.5331242084503174</v>
+        <v>0.86818379163742065</v>
       </c>
       <c r="D4" s="1">
-        <v>1.2959392070770264</v>
+        <v>1.1604779958724976</v>
       </c>
       <c r="E4" s="1">
         <v>0</v>
       </c>
       <c r="F4" s="1">
-        <v>1920000</v>
+        <v>1446966</v>
       </c>
       <c r="G4" s="1"/>
     </row>
     <row r="5">
       <c r="A5" s="1">
-        <v>0.80000001192092896</v>
+        <v>0.79000002145767212</v>
       </c>
       <c r="B5" s="1">
-        <v>0.97617626190185547</v>
+        <v>0.96912628412246704</v>
       </c>
       <c r="C5" s="1">
-        <v>2.0393087863922119</v>
+        <v>1.5331242084503174</v>
       </c>
       <c r="D5" s="1">
-        <v>1.2959392070770264</v>
+        <v>1.1604779958724976</v>
       </c>
       <c r="E5" s="1">
         <v>0</v>
       </c>
       <c r="F5" s="1">
-        <v>2386356</v>
+        <v>1920000</v>
       </c>
       <c r="G5" s="1"/>
     </row>
     <row r="6">
       <c r="A6" s="1">
-        <v>0.81000000238418579</v>
+        <v>0.80000001192092896</v>
       </c>
       <c r="B6" s="1">
-        <v>0.98930132389068604</v>
+        <v>0.97617626190185547</v>
       </c>
       <c r="C6" s="1">
-        <v>0.9121137261390686</v>
+        <v>2.0393087863922119</v>
       </c>
       <c r="D6" s="1">
-        <v>1.1024150848388672</v>
+        <v>1.1604779958724976</v>
       </c>
       <c r="E6" s="1">
         <v>0</v>
       </c>
       <c r="F6" s="1">
-        <v>2664000</v>
+        <v>2386356</v>
       </c>
       <c r="G6" s="1"/>
     </row>
     <row r="7">
       <c r="A7" s="1">
-        <v>0.81999999284744263</v>
+        <v>0.81000000238418579</v>
       </c>
       <c r="B7" s="1">
-        <v>0.98835998773574829</v>
+        <v>0.98930132389068604</v>
       </c>
       <c r="C7" s="1">
-        <v>1.292716383934021</v>
+        <v>0.9121137261390686</v>
       </c>
       <c r="D7" s="1">
         <v>1.1024150848388672</v>
@@ -2886,40 +2907,40 @@
         <v>0</v>
       </c>
       <c r="F7" s="1">
-        <v>2857800</v>
+        <v>2664000</v>
       </c>
       <c r="G7" s="1"/>
     </row>
     <row r="8">
       <c r="A8" s="1">
-        <v>0.82999998331069946</v>
+        <v>0.81999999284744263</v>
       </c>
       <c r="B8" s="1">
-        <v>0.99202698469161987</v>
+        <v>0.98835998773574829</v>
       </c>
       <c r="C8" s="1">
-        <v>0.91762042045593262</v>
+        <v>1.292716383934021</v>
       </c>
       <c r="D8" s="1">
-        <v>1.1023845672607422</v>
+        <v>1.1024150848388672</v>
       </c>
       <c r="E8" s="1">
         <v>0</v>
       </c>
       <c r="F8" s="1">
-        <v>3012852</v>
+        <v>2857800</v>
       </c>
       <c r="G8" s="1"/>
     </row>
     <row r="9">
       <c r="A9" s="1">
-        <v>0.8399999737739563</v>
+        <v>0.82999998331069946</v>
       </c>
       <c r="B9" s="1">
-        <v>0.99114120006561279</v>
+        <v>0.99202698469161987</v>
       </c>
       <c r="C9" s="1">
-        <v>0.72953236103057861</v>
+        <v>0.91762042045593262</v>
       </c>
       <c r="D9" s="1">
         <v>1.1023845672607422</v>
@@ -2928,19 +2949,19 @@
         <v>0</v>
       </c>
       <c r="F9" s="1">
-        <v>3135000</v>
+        <v>3012852</v>
       </c>
       <c r="G9" s="1"/>
     </row>
     <row r="10">
       <c r="A10" s="1">
-        <v>0.85000002384185791</v>
+        <v>0.8399999737739563</v>
       </c>
       <c r="B10" s="1">
-        <v>0.98806333541870117</v>
+        <v>0.99114120006561279</v>
       </c>
       <c r="C10" s="1">
-        <v>1.101375937461853</v>
+        <v>0.72953236103057861</v>
       </c>
       <c r="D10" s="1">
         <v>1.1023845672607422</v>
@@ -2949,19 +2970,19 @@
         <v>0</v>
       </c>
       <c r="F10" s="1">
-        <v>3293475</v>
+        <v>3135000</v>
       </c>
       <c r="G10" s="1"/>
     </row>
     <row r="11">
       <c r="A11" s="1">
-        <v>0.86000001430511475</v>
+        <v>0.85000002384185791</v>
       </c>
       <c r="B11" s="1">
-        <v>0.98938095569610596</v>
+        <v>0.98806333541870117</v>
       </c>
       <c r="C11" s="1">
-        <v>1.1986960172653198</v>
+        <v>1.101375937461853</v>
       </c>
       <c r="D11" s="1">
         <v>1.1023845672607422</v>
@@ -2970,19 +2991,19 @@
         <v>0</v>
       </c>
       <c r="F11" s="1">
-        <v>3483508.5</v>
+        <v>3293475</v>
       </c>
       <c r="G11" s="1"/>
     </row>
     <row r="12">
       <c r="A12" s="1">
-        <v>0.87000000476837158</v>
+        <v>0.86000001430511475</v>
       </c>
       <c r="B12" s="1">
-        <v>0.9917868971824646</v>
+        <v>0.98938095569610596</v>
       </c>
       <c r="C12" s="1">
-        <v>1.2237437963485718</v>
+        <v>1.1986960172653198</v>
       </c>
       <c r="D12" s="1">
         <v>1.1023845672607422</v>
@@ -2991,19 +3012,19 @@
         <v>0</v>
       </c>
       <c r="F12" s="1">
-        <v>3690240</v>
+        <v>3483508.5</v>
       </c>
       <c r="G12" s="1"/>
     </row>
     <row r="13">
       <c r="A13" s="1">
-        <v>0.87999999523162842</v>
+        <v>0.87000000476837158</v>
       </c>
       <c r="B13" s="1">
-        <v>0.9944227933883667</v>
+        <v>0.9917868971824646</v>
       </c>
       <c r="C13" s="1">
-        <v>1.1740338802337646</v>
+        <v>1.2237437963485718</v>
       </c>
       <c r="D13" s="1">
         <v>1.1023845672607422</v>
@@ -3012,19 +3033,19 @@
         <v>0</v>
       </c>
       <c r="F13" s="1">
-        <v>3953724</v>
+        <v>3690240</v>
       </c>
       <c r="G13" s="1"/>
     </row>
     <row r="14">
       <c r="A14" s="1">
-        <v>0.88999998569488525</v>
+        <v>0.87999999523162842</v>
       </c>
       <c r="B14" s="1">
-        <v>0.99644088745117188</v>
+        <v>0.9944227933883667</v>
       </c>
       <c r="C14" s="1">
-        <v>1.2190300226211548</v>
+        <v>1.1740338802337646</v>
       </c>
       <c r="D14" s="1">
         <v>1.1023845672607422</v>
@@ -3033,19 +3054,19 @@
         <v>0</v>
       </c>
       <c r="F14" s="1">
-        <v>4248024</v>
+        <v>3953724</v>
       </c>
       <c r="G14" s="1"/>
     </row>
     <row r="15">
       <c r="A15" s="1">
-        <v>0.89999997615814209</v>
+        <v>0.88999998569488525</v>
       </c>
       <c r="B15" s="1">
-        <v>0.99891406297683716</v>
+        <v>0.99644088745117188</v>
       </c>
       <c r="C15" s="1">
-        <v>1.0577876567840576</v>
+        <v>1.2190300226211548</v>
       </c>
       <c r="D15" s="1">
         <v>1.1023845672607422</v>
@@ -3054,19 +3075,19 @@
         <v>0</v>
       </c>
       <c r="F15" s="1">
-        <v>4611906</v>
+        <v>4248024</v>
       </c>
       <c r="G15" s="1"/>
     </row>
     <row r="16">
       <c r="A16" s="1">
-        <v>0.9100000262260437</v>
+        <v>0.89999997615814209</v>
       </c>
       <c r="B16" s="1">
-        <v>0.99956101179122925</v>
+        <v>0.99891406297683716</v>
       </c>
       <c r="C16" s="1">
-        <v>1.1844043731689453</v>
+        <v>1.0577876567840576</v>
       </c>
       <c r="D16" s="1">
         <v>1.1023845672607422</v>
@@ -3075,19 +3096,19 @@
         <v>0</v>
       </c>
       <c r="F16" s="1">
-        <v>5012424</v>
+        <v>4611906</v>
       </c>
       <c r="G16" s="1"/>
     </row>
     <row r="17">
       <c r="A17" s="1">
-        <v>0.92000001668930054</v>
+        <v>0.9100000262260437</v>
       </c>
       <c r="B17" s="1">
-        <v>1.0015702247619629</v>
+        <v>0.99956101179122925</v>
       </c>
       <c r="C17" s="1">
-        <v>1.0740139484405518</v>
+        <v>1.1844043731689453</v>
       </c>
       <c r="D17" s="1">
         <v>1.1023845672607422</v>
@@ -3096,19 +3117,19 @@
         <v>0</v>
       </c>
       <c r="F17" s="1">
-        <v>5510711.5</v>
+        <v>5012424</v>
       </c>
       <c r="G17" s="1"/>
     </row>
     <row r="18">
       <c r="A18" s="1">
-        <v>0.93000000715255737</v>
+        <v>0.92000001668930054</v>
       </c>
       <c r="B18" s="1">
-        <v>1.0023491382598877</v>
+        <v>1.0015702247619629</v>
       </c>
       <c r="C18" s="1">
-        <v>1.1217098236083984</v>
+        <v>1.0740139484405518</v>
       </c>
       <c r="D18" s="1">
         <v>1.1023845672607422</v>
@@ -3117,19 +3138,19 @@
         <v>0</v>
       </c>
       <c r="F18" s="1">
-        <v>6101568</v>
+        <v>5510711.5</v>
       </c>
       <c r="G18" s="1"/>
     </row>
     <row r="19">
       <c r="A19" s="1">
-        <v>0.93999999761581421</v>
+        <v>0.93000000715255737</v>
       </c>
       <c r="B19" s="1">
-        <v>1.0036189556121826</v>
+        <v>1.0023491382598877</v>
       </c>
       <c r="C19" s="1">
-        <v>1.1283949613571167</v>
+        <v>1.1217098236083984</v>
       </c>
       <c r="D19" s="1">
         <v>1.1023845672607422</v>
@@ -3138,19 +3159,19 @@
         <v>0</v>
       </c>
       <c r="F19" s="1">
-        <v>6902083.5</v>
+        <v>6101568</v>
       </c>
       <c r="G19" s="1"/>
     </row>
     <row r="20">
       <c r="A20" s="1">
-        <v>0.94999998807907104</v>
+        <v>0.93999999761581421</v>
       </c>
       <c r="B20" s="1">
-        <v>1.0049324035644531</v>
+        <v>1.0036189556121826</v>
       </c>
       <c r="C20" s="1">
-        <v>1.1756194829940796</v>
+        <v>1.1283949613571167</v>
       </c>
       <c r="D20" s="1">
         <v>1.1023845672607422</v>
@@ -3159,19 +3180,19 @@
         <v>0</v>
       </c>
       <c r="F20" s="1">
-        <v>7924414</v>
+        <v>6902083.5</v>
       </c>
       <c r="G20" s="1"/>
     </row>
     <row r="21">
       <c r="A21" s="1">
-        <v>0.95999997854232788</v>
+        <v>0.94999998807907104</v>
       </c>
       <c r="B21" s="1">
-        <v>1.006710410118103</v>
+        <v>1.0049324035644531</v>
       </c>
       <c r="C21" s="1">
-        <v>1.1274241209030151</v>
+        <v>1.1756194829940796</v>
       </c>
       <c r="D21" s="1">
         <v>1.1023845672607422</v>
@@ -3180,82 +3201,82 @@
         <v>0</v>
       </c>
       <c r="F21" s="1">
-        <v>9331798</v>
+        <v>7924414</v>
       </c>
       <c r="G21" s="1"/>
     </row>
     <row r="22">
       <c r="A22" s="1">
-        <v>0.97000002861022949</v>
+        <v>0.95999997854232788</v>
       </c>
       <c r="B22" s="1">
-        <v>1.0079548358917236</v>
+        <v>1.006710410118103</v>
       </c>
       <c r="C22" s="1">
-        <v>0.93656158447265625</v>
+        <v>1.1274241209030151</v>
       </c>
       <c r="D22" s="1">
-        <v>0.93656158447265625</v>
+        <v>1.1023845672607422</v>
       </c>
       <c r="E22" s="1">
         <v>0</v>
       </c>
       <c r="F22" s="1">
-        <v>11153564</v>
+        <v>9331798</v>
       </c>
       <c r="G22" s="1"/>
     </row>
     <row r="23">
       <c r="A23" s="1">
-        <v>0.98000001907348633</v>
+        <v>0.97000002861022949</v>
       </c>
       <c r="B23" s="1">
-        <v>1.0072263479232788</v>
+        <v>1.0079548358917236</v>
       </c>
       <c r="C23" s="1">
-        <v>0.79904496669769287</v>
+        <v>0.93656158447265625</v>
       </c>
       <c r="D23" s="1">
-        <v>0.79904496669769287</v>
+        <v>0.93656158447265625</v>
       </c>
       <c r="E23" s="1">
         <v>0</v>
       </c>
       <c r="F23" s="1">
-        <v>13789644</v>
+        <v>11153564</v>
       </c>
       <c r="G23" s="1"/>
     </row>
     <row r="24">
       <c r="A24" s="1">
-        <v>0.99000000953674316</v>
+        <v>0.98000001907348633</v>
       </c>
       <c r="B24" s="1">
-        <v>1.005123496055603</v>
+        <v>1.0072263479232788</v>
       </c>
       <c r="C24" s="1">
-        <v>0.56181508302688599</v>
+        <v>0.79904496669769287</v>
       </c>
       <c r="D24" s="1">
-        <v>0.62930065393447876</v>
+        <v>0.79904496669769287</v>
       </c>
       <c r="E24" s="1">
         <v>0</v>
       </c>
       <c r="F24" s="1">
-        <v>18968396</v>
+        <v>13789644</v>
       </c>
       <c r="G24" s="1"/>
     </row>
     <row r="25">
       <c r="A25" s="1">
-        <v>0.99099999666213989</v>
+        <v>0.99000000953674316</v>
       </c>
       <c r="B25" s="1">
-        <v>1.0046762228012085</v>
+        <v>1.005123496055603</v>
       </c>
       <c r="C25" s="1">
-        <v>0.31261944770812988</v>
+        <v>0.56181508302688599</v>
       </c>
       <c r="D25" s="1">
         <v>0.62930065393447876</v>
@@ -3264,19 +3285,19 @@
         <v>0</v>
       </c>
       <c r="F25" s="1">
-        <v>19899772</v>
+        <v>18968396</v>
       </c>
       <c r="G25" s="1"/>
     </row>
     <row r="26">
       <c r="A26" s="1">
-        <v>0.99199998378753662</v>
+        <v>0.99099999666213989</v>
       </c>
       <c r="B26" s="1">
-        <v>1.0039784908294678</v>
+        <v>1.0046762228012085</v>
       </c>
       <c r="C26" s="1">
-        <v>0.98564046621322632</v>
+        <v>0.31261944770812988</v>
       </c>
       <c r="D26" s="1">
         <v>0.62930065393447876</v>
@@ -3285,19 +3306,19 @@
         <v>0</v>
       </c>
       <c r="F26" s="1">
-        <v>20976620</v>
+        <v>19899772</v>
       </c>
       <c r="G26" s="1"/>
     </row>
     <row r="27">
       <c r="A27" s="1">
-        <v>0.99299997091293335</v>
+        <v>0.99199998378753662</v>
       </c>
       <c r="B27" s="1">
-        <v>1.003960132598877</v>
+        <v>1.0039784908294678</v>
       </c>
       <c r="C27" s="1">
-        <v>0.65712594985961914</v>
+        <v>0.98564046621322632</v>
       </c>
       <c r="D27" s="1">
         <v>0.62930065393447876</v>
@@ -3306,40 +3327,40 @@
         <v>0</v>
       </c>
       <c r="F27" s="1">
-        <v>22286994</v>
+        <v>20976620</v>
       </c>
       <c r="G27" s="1"/>
     </row>
     <row r="28">
       <c r="A28" s="1">
-        <v>0.99400001764297485</v>
+        <v>0.99299997091293335</v>
       </c>
       <c r="B28" s="1">
-        <v>1.0036110877990723</v>
+        <v>1.003960132598877</v>
       </c>
       <c r="C28" s="1">
-        <v>0.47803562879562378</v>
+        <v>0.65712594985961914</v>
       </c>
       <c r="D28" s="1">
-        <v>0.50229418277740479</v>
+        <v>0.62930065393447876</v>
       </c>
       <c r="E28" s="1">
         <v>0</v>
       </c>
       <c r="F28" s="1">
-        <v>23989048</v>
+        <v>22286994</v>
       </c>
       <c r="G28" s="1"/>
     </row>
     <row r="29">
       <c r="A29" s="1">
-        <v>0.99500000476837158</v>
+        <v>0.99400001764297485</v>
       </c>
       <c r="B29" s="1">
-        <v>1.0030828714370728</v>
+        <v>1.0036110877990723</v>
       </c>
       <c r="C29" s="1">
-        <v>0.52388936281204224</v>
+        <v>0.47803562879562378</v>
       </c>
       <c r="D29" s="1">
         <v>0.50229418277740479</v>
@@ -3348,19 +3369,19 @@
         <v>0</v>
       </c>
       <c r="F29" s="1">
-        <v>26050806</v>
+        <v>23989048</v>
       </c>
       <c r="G29" s="1"/>
     </row>
     <row r="30">
       <c r="A30" s="1">
-        <v>0.99599999189376831</v>
+        <v>0.99500000476837158</v>
       </c>
       <c r="B30" s="1">
-        <v>1.0026018619537354</v>
+        <v>1.0030828714370728</v>
       </c>
       <c r="C30" s="1">
-        <v>0.42082563042640686</v>
+        <v>0.52388936281204224</v>
       </c>
       <c r="D30" s="1">
         <v>0.50229418277740479</v>
@@ -3369,19 +3390,19 @@
         <v>0</v>
       </c>
       <c r="F30" s="1">
-        <v>28608102</v>
+        <v>26050806</v>
       </c>
       <c r="G30" s="1"/>
     </row>
     <row r="31">
       <c r="A31" s="1">
-        <v>0.99699997901916504</v>
+        <v>0.99599999189376831</v>
       </c>
       <c r="B31" s="1">
-        <v>1.0020183324813843</v>
+        <v>1.0026018619537354</v>
       </c>
       <c r="C31" s="1">
-        <v>0.58642119169235229</v>
+        <v>0.42082563042640686</v>
       </c>
       <c r="D31" s="1">
         <v>0.50229418277740479</v>
@@ -3390,58 +3411,58 @@
         <v>0</v>
       </c>
       <c r="F31" s="1">
-        <v>31666464</v>
+        <v>28608102</v>
       </c>
       <c r="G31" s="1"/>
     </row>
     <row r="32">
       <c r="A32" s="1">
-        <v>0.99800002574920654</v>
+        <v>0.99699997901916504</v>
       </c>
       <c r="B32" s="1">
-        <v>1.0016018152236938</v>
+        <v>1.0020183324813843</v>
       </c>
       <c r="C32" s="1">
-        <v>0.31947606801986694</v>
+        <v>0.58642119169235229</v>
       </c>
       <c r="D32" s="1">
-        <v>0.31947606801986694</v>
+        <v>0.50229418277740479</v>
       </c>
       <c r="E32" s="1">
         <v>0</v>
       </c>
       <c r="F32" s="1">
-        <v>36564456</v>
+        <v>31666464</v>
       </c>
       <c r="G32" s="1"/>
     </row>
     <row r="33">
       <c r="A33" s="1">
-        <v>0.99900001287460327</v>
+        <v>0.99800002574920654</v>
       </c>
       <c r="B33" s="1">
-        <v>1.0010010004043579</v>
+        <v>1.0016018152236938</v>
       </c>
       <c r="C33" s="1">
-        <v>0</v>
+        <v>0.31947606801986694</v>
       </c>
       <c r="D33" s="1">
-        <v>0.1637117862701416</v>
+        <v>0.31947606801986694</v>
       </c>
       <c r="E33" s="1">
         <v>0</v>
       </c>
       <c r="F33" s="1">
-        <v>46889656</v>
+        <v>36564456</v>
       </c>
       <c r="G33" s="1"/>
     </row>
     <row r="34">
       <c r="A34" s="1">
-        <v>0.99910002946853638</v>
+        <v>0.99900001287460327</v>
       </c>
       <c r="B34" s="1">
-        <v>1.0009007453918457</v>
+        <v>1.0010010004043579</v>
       </c>
       <c r="C34" s="1">
         <v>0</v>
@@ -3453,16 +3474,16 @@
         <v>0</v>
       </c>
       <c r="F34" s="1">
-        <v>48798384</v>
+        <v>46889656</v>
       </c>
       <c r="G34" s="1"/>
     </row>
     <row r="35">
       <c r="A35" s="1">
-        <v>0.99919998645782471</v>
+        <v>0.99910002946853638</v>
       </c>
       <c r="B35" s="1">
-        <v>1.000800609588623</v>
+        <v>1.0009007453918457</v>
       </c>
       <c r="C35" s="1">
         <v>0</v>
@@ -3474,19 +3495,19 @@
         <v>0</v>
       </c>
       <c r="F35" s="1">
-        <v>51000000</v>
+        <v>48798384</v>
       </c>
       <c r="G35" s="1"/>
     </row>
     <row r="36">
       <c r="A36" s="1">
-        <v>0.99930000305175781</v>
+        <v>0.99919998645782471</v>
       </c>
       <c r="B36" s="1">
-        <v>1.000618577003479</v>
+        <v>1.000800609588623</v>
       </c>
       <c r="C36" s="1">
-        <v>0.042846273630857468</v>
+        <v>0</v>
       </c>
       <c r="D36" s="1">
         <v>0.1637117862701416</v>
@@ -3495,19 +3516,19 @@
         <v>0</v>
       </c>
       <c r="F36" s="1">
-        <v>53597568</v>
+        <v>51000000</v>
       </c>
       <c r="G36" s="1"/>
     </row>
     <row r="37">
       <c r="A37" s="1">
-        <v>0.99940001964569092</v>
+        <v>0.99930000305175781</v>
       </c>
       <c r="B37" s="1">
-        <v>1.0005227327346802</v>
+        <v>1.000618577003479</v>
       </c>
       <c r="C37" s="1">
-        <v>0.77597999572753906</v>
+        <v>0.042846273630857468</v>
       </c>
       <c r="D37" s="1">
         <v>0.1637117862701416</v>
@@ -3516,37 +3537,37 @@
         <v>0</v>
       </c>
       <c r="F37" s="1">
-        <v>56624664</v>
+        <v>53597568</v>
       </c>
       <c r="G37" s="1"/>
     </row>
     <row r="38">
       <c r="A38" s="1">
-        <v>0.99949997663497925</v>
+        <v>0.99940001964569092</v>
       </c>
       <c r="B38" s="1">
-        <v>1.0005003213882446</v>
+        <v>1.0005227327346802</v>
       </c>
       <c r="C38" s="1">
-        <v>0</v>
+        <v>0.77597999572753906</v>
       </c>
       <c r="D38" s="1">
-        <v>0</v>
+        <v>0.1637117862701416</v>
       </c>
       <c r="E38" s="1">
         <v>0</v>
       </c>
       <c r="F38" s="1">
-        <v>60442488</v>
+        <v>56624664</v>
       </c>
       <c r="G38" s="1"/>
     </row>
     <row r="39">
       <c r="A39" s="1">
-        <v>0.99959999322891235</v>
+        <v>0.99949997663497925</v>
       </c>
       <c r="B39" s="1">
-        <v>1.000400185585022</v>
+        <v>1.0005003213882446</v>
       </c>
       <c r="C39" s="1">
         <v>0</v>
@@ -3558,16 +3579,16 @@
         <v>0</v>
       </c>
       <c r="F39" s="1">
-        <v>65539192</v>
+        <v>60442488</v>
       </c>
       <c r="G39" s="1"/>
     </row>
     <row r="40">
       <c r="A40" s="1">
-        <v>0.99970000982284546</v>
+        <v>0.99959999322891235</v>
       </c>
       <c r="B40" s="1">
-        <v>1.0003000497817993</v>
+        <v>1.000400185585022</v>
       </c>
       <c r="C40" s="1">
         <v>0</v>
@@ -3579,16 +3600,16 @@
         <v>0</v>
       </c>
       <c r="F40" s="1">
-        <v>71719624</v>
+        <v>65539192</v>
       </c>
       <c r="G40" s="1"/>
     </row>
     <row r="41">
       <c r="A41" s="1">
-        <v>0.99980002641677856</v>
+        <v>0.99970000982284546</v>
       </c>
       <c r="B41" s="1">
-        <v>1.0002000331878662</v>
+        <v>1.0003000497817993</v>
       </c>
       <c r="C41" s="1">
         <v>0</v>
@@ -3600,16 +3621,16 @@
         <v>0</v>
       </c>
       <c r="F41" s="1">
-        <v>81230648</v>
+        <v>71719624</v>
       </c>
       <c r="G41" s="1"/>
     </row>
     <row r="42">
       <c r="A42" s="1">
-        <v>0.99989998340606689</v>
+        <v>0.99980002641677856</v>
       </c>
       <c r="B42" s="1">
-        <v>1.0001000165939331</v>
+        <v>1.0002000331878662</v>
       </c>
       <c r="C42" s="1">
         <v>0</v>
@@ -3621,16 +3642,16 @@
         <v>0</v>
       </c>
       <c r="F42" s="1">
-        <v>101398784</v>
+        <v>81230648</v>
       </c>
       <c r="G42" s="1"/>
     </row>
     <row r="43">
       <c r="A43" s="1">
-        <v>0.99990999698638916</v>
+        <v>0.99989998340606689</v>
       </c>
       <c r="B43" s="1">
-        <v>1.0000900030136108</v>
+        <v>1.0001000165939331</v>
       </c>
       <c r="C43" s="1">
         <v>0</v>
@@ -3642,16 +3663,16 @@
         <v>0</v>
       </c>
       <c r="F43" s="1">
-        <v>103427008</v>
+        <v>101398784</v>
       </c>
       <c r="G43" s="1"/>
     </row>
     <row r="44">
       <c r="A44" s="1">
-        <v>0.99992001056671143</v>
+        <v>0.99990999698638916</v>
       </c>
       <c r="B44" s="1">
-        <v>1.0000799894332886</v>
+        <v>1.0000900030136108</v>
       </c>
       <c r="C44" s="1">
         <v>0</v>
@@ -3663,16 +3684,16 @@
         <v>0</v>
       </c>
       <c r="F44" s="1">
-        <v>107050672</v>
+        <v>103427008</v>
       </c>
       <c r="G44" s="1"/>
     </row>
     <row r="45">
       <c r="A45" s="1">
-        <v>0.99993002414703369</v>
+        <v>0.99992001056671143</v>
       </c>
       <c r="B45" s="1">
-        <v>1.0000699758529663</v>
+        <v>1.0000799894332886</v>
       </c>
       <c r="C45" s="1">
         <v>0</v>
@@ -3684,16 +3705,16 @@
         <v>0</v>
       </c>
       <c r="F45" s="1">
-        <v>111545632</v>
+        <v>107050672</v>
       </c>
       <c r="G45" s="1"/>
     </row>
     <row r="46">
       <c r="A46" s="1">
-        <v>0.99993997812271118</v>
+        <v>0.99993002414703369</v>
       </c>
       <c r="B46" s="1">
-        <v>1.0000600814819336</v>
+        <v>1.0000699758529663</v>
       </c>
       <c r="C46" s="1">
         <v>0</v>
@@ -3705,16 +3726,16 @@
         <v>0</v>
       </c>
       <c r="F46" s="1">
-        <v>117975472</v>
+        <v>111545632</v>
       </c>
       <c r="G46" s="1"/>
     </row>
     <row r="47">
       <c r="A47" s="1">
-        <v>0.99994999170303345</v>
+        <v>0.99993997812271118</v>
       </c>
       <c r="B47" s="1">
-        <v>1.0000500679016113</v>
+        <v>1.0000600814819336</v>
       </c>
       <c r="C47" s="1">
         <v>0</v>
@@ -3726,16 +3747,16 @@
         <v>0</v>
       </c>
       <c r="F47" s="1">
-        <v>124847136</v>
+        <v>117975472</v>
       </c>
       <c r="G47" s="1"/>
     </row>
     <row r="48">
       <c r="A48" s="1">
-        <v>0.99996000528335571</v>
+        <v>0.99994999170303345</v>
       </c>
       <c r="B48" s="1">
-        <v>1.0000400543212891</v>
+        <v>1.0000500679016113</v>
       </c>
       <c r="C48" s="1">
         <v>0</v>
@@ -3747,16 +3768,16 @@
         <v>0</v>
       </c>
       <c r="F48" s="1">
-        <v>135690928</v>
+        <v>124847136</v>
       </c>
       <c r="G48" s="1"/>
     </row>
     <row r="49">
       <c r="A49" s="1">
-        <v>0.99997001886367798</v>
+        <v>0.99996000528335571</v>
       </c>
       <c r="B49" s="1">
-        <v>1.0000300407409668</v>
+        <v>1.0000400543212891</v>
       </c>
       <c r="C49" s="1">
         <v>0</v>
@@ -3768,16 +3789,16 @@
         <v>0</v>
       </c>
       <c r="F49" s="1">
-        <v>149673344</v>
+        <v>135690928</v>
       </c>
       <c r="G49" s="1"/>
     </row>
     <row r="50">
       <c r="A50" s="1">
-        <v>0.99997997283935547</v>
+        <v>0.99997001886367798</v>
       </c>
       <c r="B50" s="1">
-        <v>1.0000200271606445</v>
+        <v>1.0000300407409668</v>
       </c>
       <c r="C50" s="1">
         <v>0</v>
@@ -3789,30 +3810,51 @@
         <v>0</v>
       </c>
       <c r="F50" s="1">
-        <v>166100704</v>
+        <v>149673344</v>
       </c>
       <c r="G50" s="1"/>
     </row>
     <row r="51">
       <c r="A51" s="1">
+        <v>0.99997997283935547</v>
+      </c>
+      <c r="B51" s="1">
+        <v>1.0000200271606445</v>
+      </c>
+      <c r="C51" s="1">
+        <v>0</v>
+      </c>
+      <c r="D51" s="1">
+        <v>0</v>
+      </c>
+      <c r="E51" s="1">
+        <v>0</v>
+      </c>
+      <c r="F51" s="1">
+        <v>166100704</v>
+      </c>
+      <c r="G51" s="1"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="1">
         <v>0.99998998641967773</v>
       </c>
-      <c r="B51" s="1">
+      <c r="B52" s="1">
         <v>1.0000100135803223</v>
       </c>
-      <c r="C51" s="1">
-        <v>0</v>
-      </c>
-      <c r="D51" s="1">
-        <v>0</v>
-      </c>
-      <c r="E51" s="1">
-        <v>0</v>
-      </c>
-      <c r="F51" s="1">
+      <c r="C52" s="1">
+        <v>0</v>
+      </c>
+      <c r="D52" s="1">
+        <v>0</v>
+      </c>
+      <c r="E52" s="1">
+        <v>0</v>
+      </c>
+      <c r="F52" s="1">
         <v>224090944</v>
       </c>
-      <c r="G51" s="1"/>
+      <c r="G52" s="1"/>
     </row>
   </sheetData>
 </worksheet>
@@ -3820,50 +3862,50 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G51"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>168</v>
+        <v>189</v>
       </c>
       <c r="B1" t="s">
-        <v>169</v>
+        <v>190</v>
       </c>
       <c r="C1" t="s">
-        <v>170</v>
+        <v>191</v>
       </c>
       <c r="D1" t="s">
-        <v>171</v>
+        <v>192</v>
       </c>
       <c r="E1" t="s">
-        <v>172</v>
+        <v>193</v>
       </c>
       <c r="F1" t="s">
-        <v>173</v>
+        <v>194</v>
       </c>
       <c r="G1" t="s">
-        <v>174</v>
+        <v>195</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1">
-        <v>0.76999998092651367</v>
+        <v>0.75999999046325684</v>
       </c>
       <c r="B2" s="1">
-        <v>0.9760587215423584</v>
+        <v>0.97962605953216553</v>
       </c>
       <c r="C2" s="1">
-        <v>0.81923800706863403</v>
+        <v>0.70494449138641357</v>
       </c>
       <c r="D2" s="1">
-        <v>1.1493052244186401</v>
+        <v>1.1231663227081299</v>
       </c>
       <c r="E2" s="1">
         <v>0</v>
       </c>
       <c r="F2" s="1">
-        <v>318300</v>
+        <v>0.11999999731779099</v>
       </c>
       <c r="G2" s="1">
         <v>0.97000002861022949</v>
@@ -3871,349 +3913,349 @@
     </row>
     <row r="3">
       <c r="A3" s="1">
-        <v>0.77999997138977051</v>
+        <v>0.76999998092651367</v>
       </c>
       <c r="B3" s="1">
-        <v>0.9740481972694397</v>
+        <v>0.9760587215423584</v>
       </c>
       <c r="C3" s="1">
-        <v>0.3026471734046936</v>
+        <v>0.81923800706863403</v>
       </c>
       <c r="D3" s="1">
-        <v>1.1493052244186401</v>
+        <v>1.1231663227081299</v>
       </c>
       <c r="E3" s="1">
         <v>0</v>
       </c>
       <c r="F3" s="1">
-        <v>1382400</v>
+        <v>318300</v>
       </c>
       <c r="G3" s="1"/>
     </row>
     <row r="4">
       <c r="A4" s="1">
-        <v>0.79000002145767212</v>
+        <v>0.77999997138977051</v>
       </c>
       <c r="B4" s="1">
-        <v>0.96554940938949585</v>
+        <v>0.9740481972694397</v>
       </c>
       <c r="C4" s="1">
-        <v>0.5191962718963623</v>
+        <v>0.3026471734046936</v>
       </c>
       <c r="D4" s="1">
-        <v>1.1493052244186401</v>
+        <v>1.1231663227081299</v>
       </c>
       <c r="E4" s="1">
         <v>0</v>
       </c>
       <c r="F4" s="1">
-        <v>1581120</v>
+        <v>1382400</v>
       </c>
       <c r="G4" s="1"/>
     </row>
     <row r="5">
       <c r="A5" s="1">
-        <v>0.80000001192092896</v>
+        <v>0.79000002145767212</v>
       </c>
       <c r="B5" s="1">
-        <v>0.95997005701065063</v>
+        <v>0.96554940938949585</v>
       </c>
       <c r="C5" s="1">
-        <v>1.7298133373260498</v>
+        <v>0.5191962718963623</v>
       </c>
       <c r="D5" s="1">
-        <v>1.1493052244186401</v>
+        <v>1.1231663227081299</v>
       </c>
       <c r="E5" s="1">
         <v>0</v>
       </c>
       <c r="F5" s="1">
-        <v>1818852</v>
+        <v>1581120</v>
       </c>
       <c r="G5" s="1"/>
     </row>
     <row r="6">
       <c r="A6" s="1">
-        <v>0.81000000238418579</v>
+        <v>0.80000001192092896</v>
       </c>
       <c r="B6" s="1">
-        <v>0.96947425603866577</v>
+        <v>0.95997005701065063</v>
       </c>
       <c r="C6" s="1">
-        <v>1.8518861532211304</v>
+        <v>1.7298133373260498</v>
       </c>
       <c r="D6" s="1">
-        <v>1.1493052244186401</v>
+        <v>1.1231663227081299</v>
       </c>
       <c r="E6" s="1">
         <v>0</v>
       </c>
       <c r="F6" s="1">
-        <v>2400000</v>
+        <v>1818852</v>
       </c>
       <c r="G6" s="1"/>
     </row>
     <row r="7">
       <c r="A7" s="1">
-        <v>0.81999999284744263</v>
+        <v>0.81000000238418579</v>
       </c>
       <c r="B7" s="1">
-        <v>0.98023539781570435</v>
+        <v>0.96947425603866577</v>
       </c>
       <c r="C7" s="1">
-        <v>1.549004077911377</v>
+        <v>1.8518861532211304</v>
       </c>
       <c r="D7" s="1">
-        <v>1.1493052244186401</v>
+        <v>1.1231663227081299</v>
       </c>
       <c r="E7" s="1">
         <v>0</v>
       </c>
       <c r="F7" s="1">
-        <v>2794491.25</v>
+        <v>2400000</v>
       </c>
       <c r="G7" s="1"/>
     </row>
     <row r="8">
       <c r="A8" s="1">
-        <v>0.82999998331069946</v>
+        <v>0.81999999284744263</v>
       </c>
       <c r="B8" s="1">
-        <v>0.98708796501159668</v>
+        <v>0.98023539781570435</v>
       </c>
       <c r="C8" s="1">
-        <v>1.1430414915084839</v>
+        <v>1.549004077911377</v>
       </c>
       <c r="D8" s="1">
-        <v>1.1493052244186401</v>
+        <v>1.1231663227081299</v>
       </c>
       <c r="E8" s="1">
         <v>0</v>
       </c>
       <c r="F8" s="1">
-        <v>3030019</v>
+        <v>2794491.25</v>
       </c>
       <c r="G8" s="1"/>
     </row>
     <row r="9">
       <c r="A9" s="1">
-        <v>0.8399999737739563</v>
+        <v>0.82999998331069946</v>
       </c>
       <c r="B9" s="1">
-        <v>0.98894459009170532</v>
+        <v>0.98708796501159668</v>
       </c>
       <c r="C9" s="1">
-        <v>0.85516160726547241</v>
+        <v>1.1430414915084839</v>
       </c>
       <c r="D9" s="1">
-        <v>1.1493052244186401</v>
+        <v>1.1231663227081299</v>
       </c>
       <c r="E9" s="1">
         <v>0</v>
       </c>
       <c r="F9" s="1">
-        <v>3238332</v>
+        <v>3030019</v>
       </c>
       <c r="G9" s="1"/>
     </row>
     <row r="10">
       <c r="A10" s="1">
-        <v>0.85000002384185791</v>
+        <v>0.8399999737739563</v>
       </c>
       <c r="B10" s="1">
-        <v>0.98737066984176636</v>
+        <v>0.98894459009170532</v>
       </c>
       <c r="C10" s="1">
-        <v>0.94048416614532471</v>
+        <v>0.85516160726547241</v>
       </c>
       <c r="D10" s="1">
-        <v>1.1493052244186401</v>
+        <v>1.1231663227081299</v>
       </c>
       <c r="E10" s="1">
         <v>0</v>
       </c>
       <c r="F10" s="1">
-        <v>3377999</v>
+        <v>3238332</v>
       </c>
       <c r="G10" s="1"/>
     </row>
     <row r="11">
       <c r="A11" s="1">
-        <v>0.86000001430511475</v>
+        <v>0.85000002384185791</v>
       </c>
       <c r="B11" s="1">
-        <v>0.98682552576065063</v>
+        <v>0.98737066984176636</v>
       </c>
       <c r="C11" s="1">
-        <v>1.2920979261398315</v>
+        <v>0.94048416614532471</v>
       </c>
       <c r="D11" s="1">
-        <v>1.1493052244186401</v>
+        <v>1.1231663227081299</v>
       </c>
       <c r="E11" s="1">
         <v>0</v>
       </c>
       <c r="F11" s="1">
-        <v>3585211</v>
+        <v>3377999</v>
       </c>
       <c r="G11" s="1"/>
     </row>
     <row r="12">
       <c r="A12" s="1">
-        <v>0.87000000476837158</v>
+        <v>0.86000001430511475</v>
       </c>
       <c r="B12" s="1">
-        <v>0.99033439159393311</v>
+        <v>0.98682552576065063</v>
       </c>
       <c r="C12" s="1">
-        <v>1.297821044921875</v>
+        <v>1.2920979261398315</v>
       </c>
       <c r="D12" s="1">
-        <v>1.1493052244186401</v>
+        <v>1.1231663227081299</v>
       </c>
       <c r="E12" s="1">
         <v>0</v>
       </c>
       <c r="F12" s="1">
-        <v>3807136</v>
+        <v>3585211</v>
       </c>
       <c r="G12" s="1"/>
     </row>
     <row r="13">
       <c r="A13" s="1">
-        <v>0.87999999523162842</v>
+        <v>0.87000000476837158</v>
       </c>
       <c r="B13" s="1">
-        <v>0.99382853507995605</v>
+        <v>0.99033439159393311</v>
       </c>
       <c r="C13" s="1">
-        <v>1.2716217041015625</v>
+        <v>1.297821044921875</v>
       </c>
       <c r="D13" s="1">
-        <v>1.1493052244186401</v>
+        <v>1.1231663227081299</v>
       </c>
       <c r="E13" s="1">
         <v>0</v>
       </c>
       <c r="F13" s="1">
-        <v>4089600</v>
+        <v>3807136</v>
       </c>
       <c r="G13" s="1"/>
     </row>
     <row r="14">
       <c r="A14" s="1">
-        <v>0.88999998569488525</v>
+        <v>0.87999999523162842</v>
       </c>
       <c r="B14" s="1">
-        <v>0.99694979190826416</v>
+        <v>0.99382853507995605</v>
       </c>
       <c r="C14" s="1">
-        <v>1.326542854309082</v>
+        <v>1.2716217041015625</v>
       </c>
       <c r="D14" s="1">
-        <v>1.1493052244186401</v>
+        <v>1.1231663227081299</v>
       </c>
       <c r="E14" s="1">
         <v>0</v>
       </c>
       <c r="F14" s="1">
-        <v>4428075</v>
+        <v>4089600</v>
       </c>
       <c r="G14" s="1"/>
     </row>
     <row r="15">
       <c r="A15" s="1">
-        <v>0.89999997615814209</v>
+        <v>0.88999998569488525</v>
       </c>
       <c r="B15" s="1">
-        <v>1.0006119012832642</v>
+        <v>0.99694979190826416</v>
       </c>
       <c r="C15" s="1">
-        <v>1.1574273109436035</v>
+        <v>1.326542854309082</v>
       </c>
       <c r="D15" s="1">
-        <v>1.1493052244186401</v>
+        <v>1.1231663227081299</v>
       </c>
       <c r="E15" s="1">
         <v>0</v>
       </c>
       <c r="F15" s="1">
-        <v>4828782</v>
+        <v>4428075</v>
       </c>
       <c r="G15" s="1"/>
     </row>
     <row r="16">
       <c r="A16" s="1">
-        <v>0.9100000262260437</v>
+        <v>0.89999997615814209</v>
       </c>
       <c r="B16" s="1">
-        <v>1.0023351907730103</v>
+        <v>1.0006119012832642</v>
       </c>
       <c r="C16" s="1">
-        <v>1.1218446493148804</v>
+        <v>1.1574273109436035</v>
       </c>
       <c r="D16" s="1">
-        <v>1.1493052244186401</v>
+        <v>1.1231663227081299</v>
       </c>
       <c r="E16" s="1">
         <v>0</v>
       </c>
       <c r="F16" s="1">
-        <v>5322523</v>
+        <v>4828782</v>
       </c>
       <c r="G16" s="1"/>
     </row>
     <row r="17">
       <c r="A17" s="1">
-        <v>0.92000001668930054</v>
+        <v>0.9100000262260437</v>
       </c>
       <c r="B17" s="1">
-        <v>1.0036342144012451</v>
+        <v>1.0023351907730103</v>
       </c>
       <c r="C17" s="1">
-        <v>1.2110621929168701</v>
+        <v>1.1218446493148804</v>
       </c>
       <c r="D17" s="1">
-        <v>1.1493052244186401</v>
+        <v>1.1231663227081299</v>
       </c>
       <c r="E17" s="1">
         <v>0</v>
       </c>
       <c r="F17" s="1">
-        <v>5896260</v>
+        <v>5322523</v>
       </c>
       <c r="G17" s="1"/>
     </row>
     <row r="18">
       <c r="A18" s="1">
-        <v>0.93000000715255737</v>
+        <v>0.92000001668930054</v>
       </c>
       <c r="B18" s="1">
-        <v>1.0058646202087402</v>
+        <v>1.0036342144012451</v>
       </c>
       <c r="C18" s="1">
-        <v>0.99048757553100586</v>
+        <v>1.2110621929168701</v>
       </c>
       <c r="D18" s="1">
-        <v>1.0669642686843872</v>
+        <v>1.1231663227081299</v>
       </c>
       <c r="E18" s="1">
         <v>0</v>
       </c>
       <c r="F18" s="1">
-        <v>6575081</v>
+        <v>5896260</v>
       </c>
       <c r="G18" s="1"/>
     </row>
     <row r="19">
       <c r="A19" s="1">
-        <v>0.93999999761581421</v>
+        <v>0.93000000715255737</v>
       </c>
       <c r="B19" s="1">
-        <v>1.005700945854187</v>
+        <v>1.0058646202087402</v>
       </c>
       <c r="C19" s="1">
-        <v>0.96551764011383057</v>
+        <v>0.99048757553100586</v>
       </c>
       <c r="D19" s="1">
         <v>1.0669642686843872</v>
@@ -4222,19 +4264,19 @@
         <v>0</v>
       </c>
       <c r="F19" s="1">
-        <v>7420857</v>
+        <v>6575081</v>
       </c>
       <c r="G19" s="1"/>
     </row>
     <row r="20">
       <c r="A20" s="1">
-        <v>0.94999998807907104</v>
+        <v>0.93999999761581421</v>
       </c>
       <c r="B20" s="1">
-        <v>1.0052779912948608</v>
+        <v>1.005700945854187</v>
       </c>
       <c r="C20" s="1">
-        <v>1.0938646793365479</v>
+        <v>0.96551764011383057</v>
       </c>
       <c r="D20" s="1">
         <v>1.0669642686843872</v>
@@ -4243,19 +4285,19 @@
         <v>0</v>
       </c>
       <c r="F20" s="1">
-        <v>8542665</v>
+        <v>7420857</v>
       </c>
       <c r="G20" s="1"/>
     </row>
     <row r="21">
       <c r="A21" s="1">
-        <v>0.95999997854232788</v>
+        <v>0.94999998807907104</v>
       </c>
       <c r="B21" s="1">
-        <v>1.0062007904052734</v>
+        <v>1.0052779912948608</v>
       </c>
       <c r="C21" s="1">
-        <v>1.2179863452911377</v>
+        <v>1.0938646793365479</v>
       </c>
       <c r="D21" s="1">
         <v>1.0669642686843872</v>
@@ -4264,61 +4306,61 @@
         <v>0</v>
       </c>
       <c r="F21" s="1">
-        <v>10054950</v>
+        <v>8542665</v>
       </c>
       <c r="G21" s="1"/>
     </row>
     <row r="22">
       <c r="A22" s="1">
-        <v>0.97000002861022949</v>
+        <v>0.95999997854232788</v>
       </c>
       <c r="B22" s="1">
-        <v>1.008384108543396</v>
+        <v>1.0062007904052734</v>
       </c>
       <c r="C22" s="1">
-        <v>0.89605551958084106</v>
+        <v>1.2179863452911377</v>
       </c>
       <c r="D22" s="1">
-        <v>0.89605551958084106</v>
+        <v>1.0669642686843872</v>
       </c>
       <c r="E22" s="1">
         <v>0</v>
       </c>
       <c r="F22" s="1">
-        <v>12047700</v>
+        <v>10054950</v>
       </c>
       <c r="G22" s="1"/>
     </row>
     <row r="23">
       <c r="A23" s="1">
-        <v>0.98000001907348633</v>
+        <v>0.97000002861022949</v>
       </c>
       <c r="B23" s="1">
-        <v>1.0072379112243652</v>
+        <v>1.008384108543396</v>
       </c>
       <c r="C23" s="1">
-        <v>0.74155145883560181</v>
+        <v>0.89605551958084106</v>
       </c>
       <c r="D23" s="1">
-        <v>0.76746970415115356</v>
+        <v>0.89605551958084106</v>
       </c>
       <c r="E23" s="1">
         <v>0</v>
       </c>
       <c r="F23" s="1">
-        <v>15048768</v>
+        <v>12047700</v>
       </c>
       <c r="G23" s="1"/>
     </row>
     <row r="24">
       <c r="A24" s="1">
-        <v>0.99000000953674316</v>
+        <v>0.98000001907348633</v>
       </c>
       <c r="B24" s="1">
-        <v>1.004554271697998</v>
+        <v>1.0072379112243652</v>
       </c>
       <c r="C24" s="1">
-        <v>0.97188836336135864</v>
+        <v>0.74155145883560181</v>
       </c>
       <c r="D24" s="1">
         <v>0.76746970415115356</v>
@@ -4327,19 +4369,19 @@
         <v>0</v>
       </c>
       <c r="F24" s="1">
-        <v>21464244</v>
+        <v>15048768</v>
       </c>
       <c r="G24" s="1"/>
     </row>
     <row r="25">
       <c r="A25" s="1">
-        <v>0.99099999666213989</v>
+        <v>0.99000000953674316</v>
       </c>
       <c r="B25" s="1">
-        <v>1.0045212507247925</v>
+        <v>1.004554271697998</v>
       </c>
       <c r="C25" s="1">
-        <v>0.82223659753799438</v>
+        <v>0.97188836336135864</v>
       </c>
       <c r="D25" s="1">
         <v>0.76746970415115356</v>
@@ -4348,40 +4390,40 @@
         <v>0</v>
       </c>
       <c r="F25" s="1">
-        <v>22670932</v>
+        <v>21464244</v>
       </c>
       <c r="G25" s="1"/>
     </row>
     <row r="26">
       <c r="A26" s="1">
-        <v>0.99199998378753662</v>
+        <v>0.99099999666213989</v>
       </c>
       <c r="B26" s="1">
-        <v>1.0043375492095947</v>
+        <v>1.0045212507247925</v>
       </c>
       <c r="C26" s="1">
-        <v>0.5350155234336853</v>
+        <v>0.82223659753799438</v>
       </c>
       <c r="D26" s="1">
-        <v>0.62261795997619629</v>
+        <v>0.76746970415115356</v>
       </c>
       <c r="E26" s="1">
         <v>0</v>
       </c>
       <c r="F26" s="1">
-        <v>24078284</v>
+        <v>22670932</v>
       </c>
       <c r="G26" s="1"/>
     </row>
     <row r="27">
       <c r="A27" s="1">
-        <v>0.99299997091293335</v>
+        <v>0.99199998378753662</v>
       </c>
       <c r="B27" s="1">
-        <v>1.0038648843765259</v>
+        <v>1.0043375492095947</v>
       </c>
       <c r="C27" s="1">
-        <v>0.63121283054351807</v>
+        <v>0.5350155234336853</v>
       </c>
       <c r="D27" s="1">
         <v>0.62261795997619629</v>
@@ -4390,19 +4432,19 @@
         <v>0</v>
       </c>
       <c r="F27" s="1">
-        <v>25756350</v>
+        <v>24078284</v>
       </c>
       <c r="G27" s="1"/>
     </row>
     <row r="28">
       <c r="A28" s="1">
-        <v>0.99400001764297485</v>
+        <v>0.99299997091293335</v>
       </c>
       <c r="B28" s="1">
-        <v>1.0034899711608887</v>
+        <v>1.0038648843765259</v>
       </c>
       <c r="C28" s="1">
-        <v>0.70162492990493774</v>
+        <v>0.63121283054351807</v>
       </c>
       <c r="D28" s="1">
         <v>0.62261795997619629</v>
@@ -4411,61 +4453,61 @@
         <v>0</v>
       </c>
       <c r="F28" s="1">
-        <v>27843632</v>
+        <v>25756350</v>
       </c>
       <c r="G28" s="1"/>
     </row>
     <row r="29">
       <c r="A29" s="1">
-        <v>0.99500000476837158</v>
+        <v>0.99400001764297485</v>
       </c>
       <c r="B29" s="1">
-        <v>1.0031867027282715</v>
+        <v>1.0034899711608887</v>
       </c>
       <c r="C29" s="1">
-        <v>0.49240928888320923</v>
+        <v>0.70162492990493774</v>
       </c>
       <c r="D29" s="1">
-        <v>0.49240928888320923</v>
+        <v>0.62261795997619629</v>
       </c>
       <c r="E29" s="1">
         <v>0</v>
       </c>
       <c r="F29" s="1">
-        <v>30081252</v>
+        <v>27843632</v>
       </c>
       <c r="G29" s="1"/>
     </row>
     <row r="30">
       <c r="A30" s="1">
-        <v>0.99599999189376831</v>
+        <v>0.99500000476837158</v>
       </c>
       <c r="B30" s="1">
-        <v>1.002673864364624</v>
+        <v>1.0031867027282715</v>
       </c>
       <c r="C30" s="1">
-        <v>0.38748350739479065</v>
+        <v>0.49240928888320923</v>
       </c>
       <c r="D30" s="1">
-        <v>0.39862799644470215</v>
+        <v>0.49240928888320923</v>
       </c>
       <c r="E30" s="1">
         <v>0</v>
       </c>
       <c r="F30" s="1">
-        <v>32840572</v>
+        <v>30081252</v>
       </c>
       <c r="G30" s="1"/>
     </row>
     <row r="31">
       <c r="A31" s="1">
-        <v>0.99699997901916504</v>
+        <v>0.99599999189376831</v>
       </c>
       <c r="B31" s="1">
-        <v>1.0020568370819092</v>
+        <v>1.002673864364624</v>
       </c>
       <c r="C31" s="1">
-        <v>0.36266124248504639</v>
+        <v>0.38748350739479065</v>
       </c>
       <c r="D31" s="1">
         <v>0.39862799644470215</v>
@@ -4474,19 +4516,19 @@
         <v>0</v>
       </c>
       <c r="F31" s="1">
-        <v>36368820</v>
+        <v>32840572</v>
       </c>
       <c r="G31" s="1"/>
     </row>
     <row r="32">
       <c r="A32" s="1">
-        <v>0.99800002574920654</v>
+        <v>0.99699997901916504</v>
       </c>
       <c r="B32" s="1">
-        <v>1.0014160871505737</v>
+        <v>1.0020568370819092</v>
       </c>
       <c r="C32" s="1">
-        <v>0.38896730542182922</v>
+        <v>0.36266124248504639</v>
       </c>
       <c r="D32" s="1">
         <v>0.39862799644470215</v>
@@ -4495,19 +4537,19 @@
         <v>0</v>
       </c>
       <c r="F32" s="1">
-        <v>42322680</v>
+        <v>36368820</v>
       </c>
       <c r="G32" s="1"/>
     </row>
     <row r="33">
       <c r="A33" s="1">
-        <v>0.99900001287460327</v>
+        <v>0.99800002574920654</v>
       </c>
       <c r="B33" s="1">
-        <v>1.0008029937744141</v>
+        <v>1.0014160871505737</v>
       </c>
       <c r="C33" s="1">
-        <v>0.27975207567214966</v>
+        <v>0.38896730542182922</v>
       </c>
       <c r="D33" s="1">
         <v>0.39862799644470215</v>
@@ -4516,19 +4558,19 @@
         <v>0</v>
       </c>
       <c r="F33" s="1">
-        <v>54880188</v>
+        <v>42322680</v>
       </c>
       <c r="G33" s="1"/>
     </row>
     <row r="34">
       <c r="A34" s="1">
-        <v>0.99910002946853638</v>
+        <v>0.99900001287460327</v>
       </c>
       <c r="B34" s="1">
-        <v>1.0007308721542358</v>
+        <v>1.0008029937744141</v>
       </c>
       <c r="C34" s="1">
-        <v>0.046653147786855698</v>
+        <v>0.27975207567214966</v>
       </c>
       <c r="D34" s="1">
         <v>0.39862799644470215</v>
@@ -4537,19 +4579,19 @@
         <v>0</v>
       </c>
       <c r="F34" s="1">
-        <v>56840024</v>
+        <v>54880188</v>
       </c>
       <c r="G34" s="1"/>
     </row>
     <row r="35">
       <c r="A35" s="1">
-        <v>0.99919998645782471</v>
+        <v>0.99910002946853638</v>
       </c>
       <c r="B35" s="1">
-        <v>1.0006353855133057</v>
+        <v>1.0007308721542358</v>
       </c>
       <c r="C35" s="1">
-        <v>1.4369083642959595</v>
+        <v>0.046653147786855698</v>
       </c>
       <c r="D35" s="1">
         <v>0.39862799644470215</v>
@@ -4558,37 +4600,37 @@
         <v>0</v>
       </c>
       <c r="F35" s="1">
-        <v>59264676</v>
+        <v>56840024</v>
       </c>
       <c r="G35" s="1"/>
     </row>
     <row r="36">
       <c r="A36" s="1">
-        <v>0.99930000305175781</v>
+        <v>0.99919998645782471</v>
       </c>
       <c r="B36" s="1">
-        <v>1.0007004737854004</v>
+        <v>1.0006353855133057</v>
       </c>
       <c r="C36" s="1">
-        <v>0</v>
+        <v>1.4369083642959595</v>
       </c>
       <c r="D36" s="1">
-        <v>0.035682540386915207</v>
+        <v>0.39862799644470215</v>
       </c>
       <c r="E36" s="1">
         <v>0</v>
       </c>
       <c r="F36" s="1">
-        <v>61777728</v>
+        <v>59264676</v>
       </c>
       <c r="G36" s="1"/>
     </row>
     <row r="37">
       <c r="A37" s="1">
-        <v>0.99940001964569092</v>
+        <v>0.99930000305175781</v>
       </c>
       <c r="B37" s="1">
-        <v>1.0006003379821777</v>
+        <v>1.0007004737854004</v>
       </c>
       <c r="C37" s="1">
         <v>0</v>
@@ -4600,16 +4642,16 @@
         <v>0</v>
       </c>
       <c r="F37" s="1">
-        <v>65098296</v>
+        <v>61777728</v>
       </c>
       <c r="G37" s="1"/>
     </row>
     <row r="38">
       <c r="A38" s="1">
-        <v>0.99949997663497925</v>
+        <v>0.99940001964569092</v>
       </c>
       <c r="B38" s="1">
-        <v>1.0005003213882446</v>
+        <v>1.0006003379821777</v>
       </c>
       <c r="C38" s="1">
         <v>0</v>
@@ -4621,16 +4663,16 @@
         <v>0</v>
       </c>
       <c r="F38" s="1">
-        <v>68856104</v>
+        <v>65098296</v>
       </c>
       <c r="G38" s="1"/>
     </row>
     <row r="39">
       <c r="A39" s="1">
-        <v>0.99959999322891235</v>
+        <v>0.99949997663497925</v>
       </c>
       <c r="B39" s="1">
-        <v>1.000400185585022</v>
+        <v>1.0005003213882446</v>
       </c>
       <c r="C39" s="1">
         <v>0</v>
@@ -4642,16 +4684,16 @@
         <v>0</v>
       </c>
       <c r="F39" s="1">
-        <v>74008312</v>
+        <v>68856104</v>
       </c>
       <c r="G39" s="1"/>
     </row>
     <row r="40">
       <c r="A40" s="1">
-        <v>0.99970000982284546</v>
+        <v>0.99959999322891235</v>
       </c>
       <c r="B40" s="1">
-        <v>1.0003000497817993</v>
+        <v>1.000400185585022</v>
       </c>
       <c r="C40" s="1">
         <v>0</v>
@@ -4663,19 +4705,19 @@
         <v>0</v>
       </c>
       <c r="F40" s="1">
-        <v>81060160</v>
+        <v>74008312</v>
       </c>
       <c r="G40" s="1"/>
     </row>
     <row r="41">
       <c r="A41" s="1">
-        <v>0.99980002641677856</v>
+        <v>0.99970000982284546</v>
       </c>
       <c r="B41" s="1">
-        <v>1.0001785755157471</v>
+        <v>1.0003000497817993</v>
       </c>
       <c r="C41" s="1">
-        <v>0.2141803503036499</v>
+        <v>0</v>
       </c>
       <c r="D41" s="1">
         <v>0.035682540386915207</v>
@@ -4684,37 +4726,37 @@
         <v>0</v>
       </c>
       <c r="F41" s="1">
-        <v>91315736</v>
+        <v>81060160</v>
       </c>
       <c r="G41" s="1"/>
     </row>
     <row r="42">
       <c r="A42" s="1">
-        <v>0.99989998340606689</v>
+        <v>0.99980002641677856</v>
       </c>
       <c r="B42" s="1">
-        <v>1.0001000165939331</v>
+        <v>1.0001785755157471</v>
       </c>
       <c r="C42" s="1">
-        <v>0</v>
+        <v>0.2141803503036499</v>
       </c>
       <c r="D42" s="1">
-        <v>0</v>
+        <v>0.035682540386915207</v>
       </c>
       <c r="E42" s="1">
         <v>0</v>
       </c>
       <c r="F42" s="1">
-        <v>110657360</v>
+        <v>91315736</v>
       </c>
       <c r="G42" s="1"/>
     </row>
     <row r="43">
       <c r="A43" s="1">
-        <v>0.99990999698638916</v>
+        <v>0.99989998340606689</v>
       </c>
       <c r="B43" s="1">
-        <v>1.0000900030136108</v>
+        <v>1.0001000165939331</v>
       </c>
       <c r="C43" s="1">
         <v>0</v>
@@ -4726,16 +4768,16 @@
         <v>0</v>
       </c>
       <c r="F43" s="1">
-        <v>114144000</v>
+        <v>110657360</v>
       </c>
       <c r="G43" s="1"/>
     </row>
     <row r="44">
       <c r="A44" s="1">
-        <v>0.99992001056671143</v>
+        <v>0.99990999698638916</v>
       </c>
       <c r="B44" s="1">
-        <v>1.0000799894332886</v>
+        <v>1.0000900030136108</v>
       </c>
       <c r="C44" s="1">
         <v>0</v>
@@ -4747,16 +4789,16 @@
         <v>0</v>
       </c>
       <c r="F44" s="1">
-        <v>117563520</v>
+        <v>114144000</v>
       </c>
       <c r="G44" s="1"/>
     </row>
     <row r="45">
       <c r="A45" s="1">
-        <v>0.99993002414703369</v>
+        <v>0.99992001056671143</v>
       </c>
       <c r="B45" s="1">
-        <v>1.0000699758529663</v>
+        <v>1.0000799894332886</v>
       </c>
       <c r="C45" s="1">
         <v>0</v>
@@ -4768,16 +4810,16 @@
         <v>0</v>
       </c>
       <c r="F45" s="1">
-        <v>122471040</v>
+        <v>117563520</v>
       </c>
       <c r="G45" s="1"/>
     </row>
     <row r="46">
       <c r="A46" s="1">
-        <v>0.99993997812271118</v>
+        <v>0.99993002414703369</v>
       </c>
       <c r="B46" s="1">
-        <v>1.0000600814819336</v>
+        <v>1.0000699758529663</v>
       </c>
       <c r="C46" s="1">
         <v>0</v>
@@ -4789,16 +4831,16 @@
         <v>0</v>
       </c>
       <c r="F46" s="1">
-        <v>128148000</v>
+        <v>122471040</v>
       </c>
       <c r="G46" s="1"/>
     </row>
     <row r="47">
       <c r="A47" s="1">
-        <v>0.99994999170303345</v>
+        <v>0.99993997812271118</v>
       </c>
       <c r="B47" s="1">
-        <v>1.0000500679016113</v>
+        <v>1.0000600814819336</v>
       </c>
       <c r="C47" s="1">
         <v>0</v>
@@ -4810,16 +4852,16 @@
         <v>0</v>
       </c>
       <c r="F47" s="1">
-        <v>135058304</v>
+        <v>128148000</v>
       </c>
       <c r="G47" s="1"/>
     </row>
     <row r="48">
       <c r="A48" s="1">
-        <v>0.99996000528335571</v>
+        <v>0.99994999170303345</v>
       </c>
       <c r="B48" s="1">
-        <v>1.0000400543212891</v>
+        <v>1.0000500679016113</v>
       </c>
       <c r="C48" s="1">
         <v>0</v>
@@ -4831,16 +4873,16 @@
         <v>0</v>
       </c>
       <c r="F48" s="1">
-        <v>143498640</v>
+        <v>135058304</v>
       </c>
       <c r="G48" s="1"/>
     </row>
     <row r="49">
       <c r="A49" s="1">
-        <v>0.99997001886367798</v>
+        <v>0.99996000528335571</v>
       </c>
       <c r="B49" s="1">
-        <v>1.0000300407409668</v>
+        <v>1.0000400543212891</v>
       </c>
       <c r="C49" s="1">
         <v>0</v>
@@ -4852,16 +4894,16 @@
         <v>0</v>
       </c>
       <c r="F49" s="1">
-        <v>154964256</v>
+        <v>143498640</v>
       </c>
       <c r="G49" s="1"/>
     </row>
     <row r="50">
       <c r="A50" s="1">
-        <v>0.99997997283935547</v>
+        <v>0.99997001886367798</v>
       </c>
       <c r="B50" s="1">
-        <v>1.0000200271606445</v>
+        <v>1.0000300407409668</v>
       </c>
       <c r="C50" s="1">
         <v>0</v>
@@ -4873,30 +4915,51 @@
         <v>0</v>
       </c>
       <c r="F50" s="1">
-        <v>177060464</v>
+        <v>154964256</v>
       </c>
       <c r="G50" s="1"/>
     </row>
     <row r="51">
       <c r="A51" s="1">
+        <v>0.99997997283935547</v>
+      </c>
+      <c r="B51" s="1">
+        <v>1.0000200271606445</v>
+      </c>
+      <c r="C51" s="1">
+        <v>0</v>
+      </c>
+      <c r="D51" s="1">
+        <v>0</v>
+      </c>
+      <c r="E51" s="1">
+        <v>0</v>
+      </c>
+      <c r="F51" s="1">
+        <v>177060464</v>
+      </c>
+      <c r="G51" s="1"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="1">
         <v>0.99998998641967773</v>
       </c>
-      <c r="B51" s="1">
+      <c r="B52" s="1">
         <v>1.0000100135803223</v>
       </c>
-      <c r="C51" s="1">
-        <v>0</v>
-      </c>
-      <c r="D51" s="1">
-        <v>0</v>
-      </c>
-      <c r="E51" s="1">
-        <v>0</v>
-      </c>
-      <c r="F51" s="1">
+      <c r="C52" s="1">
+        <v>0</v>
+      </c>
+      <c r="D52" s="1">
+        <v>0</v>
+      </c>
+      <c r="E52" s="1">
+        <v>0</v>
+      </c>
+      <c r="F52" s="1">
         <v>223548672</v>
       </c>
-      <c r="G51" s="1"/>
+      <c r="G52" s="1"/>
     </row>
   </sheetData>
 </worksheet>
@@ -4909,25 +4972,25 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>175</v>
+        <v>189</v>
       </c>
       <c r="B1" t="s">
-        <v>176</v>
+        <v>190</v>
       </c>
       <c r="C1" t="s">
-        <v>177</v>
+        <v>191</v>
       </c>
       <c r="D1" t="s">
-        <v>178</v>
+        <v>192</v>
       </c>
       <c r="E1" t="s">
-        <v>179</v>
+        <v>193</v>
       </c>
       <c r="F1" t="s">
-        <v>180</v>
+        <v>194</v>
       </c>
       <c r="G1" t="s">
-        <v>181</v>
+        <v>195</v>
       </c>
     </row>
     <row r="2">
@@ -5231,7 +5294,7 @@
         <v>0.88999998569488525</v>
       </c>
       <c r="B16" s="1">
-        <v>1.0008316040039063</v>
+        <v>1.0008316040039062</v>
       </c>
       <c r="C16" s="1">
         <v>1.1997040510177612</v>
@@ -6035,25 +6098,25 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>182</v>
+        <v>189</v>
       </c>
       <c r="B1" t="s">
-        <v>183</v>
+        <v>190</v>
       </c>
       <c r="C1" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="D1" t="s">
-        <v>185</v>
+        <v>192</v>
       </c>
       <c r="E1" t="s">
-        <v>186</v>
+        <v>193</v>
       </c>
       <c r="F1" t="s">
-        <v>187</v>
+        <v>194</v>
       </c>
       <c r="G1" t="s">
-        <v>188</v>
+        <v>195</v>
       </c>
     </row>
     <row r="2">

</xml_diff>